<commit_message>
Add protocol extras to household and tracking checks, and update configuration files
- Integrated `run_household_protocol` and `run_tracking_protocol` functions to extend issue reporting capabilities in household.py and tracking.py.
- Updated household_columns.yaml with new duration and transport eligibility parameters.
- Enhanced tracking_columns.yaml with additional fields for duplicate phone handling and girl contact information.
- Modified error log files to reflect changes in data structure.
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,188 +464,188 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Samara</t>
+          <t>Shazia begum</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>373658</v>
+        <v>373696</v>
       </c>
       <c r="C3" t="n">
-        <v>33</v>
+        <v>120</v>
       </c>
       <c r="D3" t="n">
-        <v>22</v>
+        <v>100</v>
       </c>
       <c r="E3" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Kainat</t>
+          <t>Irum Ikram</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>373712</v>
+        <v>373642</v>
       </c>
       <c r="C4" t="n">
-        <v>27</v>
+        <v>104</v>
       </c>
       <c r="D4" t="n">
-        <v>18</v>
+        <v>97</v>
       </c>
       <c r="E4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Alia Khan</t>
+          <t>Shafaq Zahra</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>373681</v>
+        <v>373646</v>
       </c>
       <c r="C5" t="n">
-        <v>23</v>
+        <v>104</v>
       </c>
       <c r="D5" t="n">
-        <v>18</v>
+        <v>96</v>
       </c>
       <c r="E5" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>373692</v>
+        <v>373648</v>
       </c>
       <c r="C6" t="n">
-        <v>20</v>
+        <v>111</v>
       </c>
       <c r="D6" t="n">
-        <v>18</v>
+        <v>87</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Summiya Hayat</t>
+          <t>Asma Bibi</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>373710</v>
+        <v>373641</v>
       </c>
       <c r="C7" t="n">
+        <v>106</v>
+      </c>
+      <c r="D7" t="n">
+        <v>85</v>
+      </c>
+      <c r="E7" t="n">
         <v>21</v>
-      </c>
-      <c r="D7" t="n">
-        <v>10</v>
-      </c>
-      <c r="E7" t="n">
-        <v>11</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Rehana Bibi</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>373691</v>
+        <v>373684</v>
       </c>
       <c r="C8" t="n">
-        <v>13</v>
+        <v>178</v>
       </c>
       <c r="D8" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Naureen</t>
+          <t>Sadia Rustum</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>884887</v>
+        <v>373649</v>
       </c>
       <c r="C9" t="n">
-        <v>12</v>
+        <v>87</v>
       </c>
       <c r="D9" t="n">
-        <v>10</v>
+        <v>72</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sajjad Khan</t>
+          <t>Muhammad Yousaf</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>373700</v>
+        <v>373690</v>
       </c>
       <c r="C10" t="n">
+        <v>72</v>
+      </c>
+      <c r="D10" t="n">
+        <v>64</v>
+      </c>
+      <c r="E10" t="n">
         <v>8</v>
-      </c>
-      <c r="D10" t="n">
-        <v>8</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Muhammad naeem</t>
+          <t>Jaweria</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>571571</v>
+        <v>163495</v>
       </c>
       <c r="C11" t="n">
-        <v>16</v>
+        <v>57</v>
       </c>
       <c r="D11" t="n">
-        <v>7</v>
+        <v>56</v>
       </c>
       <c r="E11" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Zain Ul Abideen</t>
+          <t>Naureen Khan</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>373667</v>
+        <v>373716</v>
       </c>
       <c r="C12" t="n">
-        <v>6</v>
+        <v>48</v>
       </c>
       <c r="D12" t="n">
-        <v>6</v>
+        <v>48</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
@@ -654,93 +654,93 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Mahnoor</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373646</v>
+        <v>373705</v>
       </c>
       <c r="C13" t="n">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="D13" t="n">
+        <v>47</v>
+      </c>
+      <c r="E13" t="n">
         <v>4</v>
-      </c>
-      <c r="E13" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Javairia</t>
+          <t>Furqan Ullah Khan</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>373651</v>
+        <v>373683</v>
       </c>
       <c r="C14" t="n">
+        <v>55</v>
+      </c>
+      <c r="D14" t="n">
+        <v>46</v>
+      </c>
+      <c r="E14" t="n">
         <v>9</v>
-      </c>
-      <c r="D14" t="n">
-        <v>4</v>
-      </c>
-      <c r="E14" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Hijab Zahra</t>
+          <t>Bushra Ayub</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373637</v>
+        <v>373671</v>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>51</v>
       </c>
       <c r="D15" t="n">
-        <v>4</v>
+        <v>46</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Muniba Shamim</t>
+          <t>Khalida Bibi</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>373659</v>
+        <v>373673</v>
       </c>
       <c r="C16" t="n">
-        <v>18</v>
+        <v>50</v>
       </c>
       <c r="D16" t="n">
-        <v>2</v>
+        <v>46</v>
       </c>
       <c r="E16" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Furqan Ullah Khan</t>
+          <t>Asma Gull</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>373683</v>
+        <v>373672</v>
       </c>
       <c r="C17" t="n">
-        <v>10</v>
+        <v>53</v>
       </c>
       <c r="D17" t="n">
-        <v>2</v>
+        <v>45</v>
       </c>
       <c r="E17" t="n">
         <v>8</v>
@@ -749,302 +749,302 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Asma Gull</t>
+          <t>Laiba Shams</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>373672</v>
+        <v>373706</v>
       </c>
       <c r="C18" t="n">
-        <v>9</v>
+        <v>42</v>
       </c>
       <c r="D18" t="n">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="E18" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Bushra Ayub</t>
+          <t>Javairia</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>373671</v>
+        <v>373651</v>
       </c>
       <c r="C19" t="n">
-        <v>7</v>
+        <v>39</v>
       </c>
       <c r="D19" t="n">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="E19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Syed Haider Abbas</t>
+          <t>Lati Khan</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>373713</v>
+        <v>373665</v>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="D20" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Shazia begum</t>
+          <t>Summiya Hayat</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>373696</v>
+        <v>373710</v>
       </c>
       <c r="C21" t="n">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="D21" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="E21" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Laiba Shams</t>
+          <t>Naureen</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>373706</v>
+        <v>884887</v>
       </c>
       <c r="C22" t="n">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="D22" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="E22" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Laiba Khan</t>
+          <t>Muniba Shamim</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>373653</v>
+        <v>373659</v>
       </c>
       <c r="C23" t="n">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Mahnoorr</t>
+          <t>Munawar Khan</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>373670</v>
+        <v>373668</v>
       </c>
       <c r="C24" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="D24" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E24" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Samreen</t>
+          <t>Lati Khan</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>639258</v>
+        <v>564273</v>
       </c>
       <c r="C25" t="n">
+        <v>21</v>
+      </c>
+      <c r="D25" t="n">
+        <v>20</v>
+      </c>
+      <c r="E25" t="n">
         <v>1</v>
-      </c>
-      <c r="D25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Mehran Khan</t>
+          <t>Lati khan</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>373684</v>
+        <v>671211</v>
       </c>
       <c r="C26" t="n">
-        <v>97</v>
+        <v>19</v>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E26" t="n">
-        <v>97</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Naureen khan</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>373648</v>
+        <v>453925</v>
       </c>
       <c r="C27" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="E27" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Asma Bibi</t>
+          <t>Kainat</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>373641</v>
+        <v>373712</v>
       </c>
       <c r="C28" t="n">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="D28" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E28" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Sadia Rustum</t>
+          <t>Zohra</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>373649</v>
+        <v>373692</v>
       </c>
       <c r="C29" t="n">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="D29" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="E29" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Chashm Gul</t>
+          <t>Anum Gul</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>373695</v>
+        <v>373656</v>
       </c>
       <c r="C30" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="E30" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Samara</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>373642</v>
+        <v>373658</v>
       </c>
       <c r="C31" t="n">
-        <v>7</v>
+        <v>47</v>
       </c>
       <c r="D31" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="E31" t="n">
-        <v>7</v>
+        <v>36</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Muhammad Yousaf</t>
+          <t>Rehana Bibi</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>373690</v>
+        <v>373691</v>
       </c>
       <c r="C32" t="n">
+        <v>34</v>
+      </c>
+      <c r="D32" t="n">
         <v>7</v>
       </c>
-      <c r="D32" t="n">
-        <v>0</v>
-      </c>
       <c r="E32" t="n">
-        <v>7</v>
+        <v>27</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Anum Gul</t>
+          <t>Alia Khan</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>373656</v>
+        <v>373681</v>
       </c>
       <c r="C33" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="D33" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E33" t="n">
         <v>5</v>
@@ -1053,36 +1053,36 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Khalida Bibi</t>
+          <t>Ishaq Khan</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>373673</v>
+        <v>373699</v>
       </c>
       <c r="C34" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Mahnoor</t>
+          <t>Laiba Khan</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>373705</v>
+        <v>373653</v>
       </c>
       <c r="C35" t="n">
+        <v>8</v>
+      </c>
+      <c r="D35" t="n">
         <v>4</v>
-      </c>
-      <c r="D35" t="n">
-        <v>0</v>
       </c>
       <c r="E35" t="n">
         <v>4</v>
@@ -1091,182 +1091,182 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Ishaq Khan</t>
+          <t>Nazia</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>373699</v>
+        <v>373657</v>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D36" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E36" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Lati Khan</t>
+          <t>Nillum Bibi</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>373665</v>
+        <v>373652</v>
       </c>
       <c r="C37" t="n">
+        <v>8</v>
+      </c>
+      <c r="D37" t="n">
         <v>3</v>
       </c>
-      <c r="D37" t="n">
-        <v>0</v>
-      </c>
       <c r="E37" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Muhammad Naeem</t>
+          <t>Zain Ul Abideen</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>373694</v>
+        <v>373667</v>
       </c>
       <c r="C38" t="n">
         <v>3</v>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E38" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Nillum Bibi</t>
+          <t>Muhammad Noor</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>373652</v>
+        <v>373701</v>
       </c>
       <c r="C39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Munawar Khan</t>
+          <t>Muhammad Shahid Khan</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>373668</v>
+        <v>373662</v>
       </c>
       <c r="C40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E40" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Shehla Noor</t>
+          <t>Chashm Gul</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>373650</v>
+        <v>373695</v>
       </c>
       <c r="C41" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D41" t="n">
         <v>0</v>
       </c>
       <c r="E41" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Jaweria</t>
+          <t>Muhammad naeem</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>163495</v>
+        <v>571571</v>
       </c>
       <c r="C42" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D42" t="n">
         <v>0</v>
       </c>
       <c r="E42" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Lati Khan</t>
+          <t>Muhammad Naeem</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>564273</v>
+        <v>373694</v>
       </c>
       <c r="C43" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D43" t="n">
         <v>0</v>
       </c>
       <c r="E43" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Muhammad Noor</t>
+          <t>Shehla Noor</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>373701</v>
+        <v>373650</v>
       </c>
       <c r="C44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D44" t="n">
         <v>0</v>
       </c>
       <c r="E44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Sidra Khan</t>
+          <t>Aisha Aman</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>373645</v>
+        <v>373704</v>
       </c>
       <c r="C45" t="n">
         <v>1</v>
@@ -1275,6 +1275,82 @@
         <v>0</v>
       </c>
       <c r="E45" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Mahnoorr</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>373670</v>
+      </c>
+      <c r="C46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Rahila Naaz</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>373715</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Robina Shaheen</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>373639</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Sidra Khan</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>373645</v>
+      </c>
+      <c r="C49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1342,29 +1418,29 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sajjad Khan</t>
+          <t>Naureen khan</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>373700</v>
+        <v>453925</v>
       </c>
       <c r="C2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="E2" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>100</v>
+        <v>900</v>
       </c>
       <c r="H2" t="n">
-        <v>100</v>
+        <v>900</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -1373,60 +1449,60 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Hijab Zahra</t>
+          <t>Lati Khan</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>373637</v>
+        <v>564273</v>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>100</v>
+        <v>233.33</v>
       </c>
       <c r="H3" t="n">
-        <v>100</v>
+        <v>222.22</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>11.11</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Syed Haider Abbas</t>
+          <t>Lati khan</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>373713</v>
+        <v>671211</v>
       </c>
       <c r="C4" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>100</v>
+        <v>211.11</v>
       </c>
       <c r="H4" t="n">
-        <v>100</v>
+        <v>211.11</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -1435,776 +1511,776 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Samreen</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>639258</v>
+        <v>373684</v>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>134</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>178</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>79</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="G5" t="n">
-        <v>100</v>
+        <v>132.84</v>
       </c>
       <c r="H5" t="n">
-        <v>100</v>
+        <v>58.96</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>73.88</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Mehran Khan</t>
+          <t>Naureen Khan</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>373684</v>
+        <v>373716</v>
       </c>
       <c r="C6" t="n">
-        <v>134</v>
+        <v>53</v>
       </c>
       <c r="D6" t="n">
-        <v>97</v>
+        <v>48</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="F6" t="n">
-        <v>97</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>72.39</v>
+        <v>90.56999999999999</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>90.56999999999999</v>
       </c>
       <c r="I6" t="n">
-        <v>72.39</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Muhammad Naeem</t>
+          <t>Shazia begum</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>373694</v>
+        <v>373696</v>
       </c>
       <c r="C7" t="n">
-        <v>6</v>
+        <v>141</v>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>120</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="F7" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="G7" t="n">
-        <v>50</v>
+        <v>85.11</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>70.92</v>
       </c>
       <c r="I7" t="n">
-        <v>50</v>
+        <v>14.18</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Shehla Noor</t>
+          <t>Sadia Rustum</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>373650</v>
+        <v>373649</v>
       </c>
       <c r="C8" t="n">
-        <v>4</v>
+        <v>103</v>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>87</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="F8" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="G8" t="n">
-        <v>50</v>
+        <v>84.47</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="I8" t="n">
-        <v>50</v>
+        <v>14.56</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Zain Ul Abideen</t>
+          <t>Jaweria</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>373667</v>
+        <v>163495</v>
       </c>
       <c r="C9" t="n">
-        <v>13</v>
+        <v>68</v>
       </c>
       <c r="D9" t="n">
-        <v>6</v>
+        <v>57</v>
       </c>
       <c r="E9" t="n">
-        <v>6</v>
+        <v>56</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>46.15</v>
+        <v>83.81999999999999</v>
       </c>
       <c r="H9" t="n">
-        <v>46.15</v>
+        <v>82.34999999999999</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>1.47</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Samara</t>
+          <t>Shafaq Zahra</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>373658</v>
+        <v>373646</v>
       </c>
       <c r="C10" t="n">
-        <v>73</v>
+        <v>126</v>
       </c>
       <c r="D10" t="n">
-        <v>33</v>
+        <v>104</v>
       </c>
       <c r="E10" t="n">
-        <v>22</v>
+        <v>96</v>
       </c>
       <c r="F10" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="G10" t="n">
-        <v>45.21</v>
+        <v>82.54000000000001</v>
       </c>
       <c r="H10" t="n">
-        <v>30.14</v>
+        <v>76.19</v>
       </c>
       <c r="I10" t="n">
-        <v>15.07</v>
+        <v>6.35</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Kainat</t>
+          <t>Asma Bibi</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>373712</v>
+        <v>373641</v>
       </c>
       <c r="C11" t="n">
-        <v>60</v>
+        <v>129</v>
       </c>
       <c r="D11" t="n">
-        <v>27</v>
+        <v>106</v>
       </c>
       <c r="E11" t="n">
-        <v>18</v>
+        <v>85</v>
       </c>
       <c r="F11" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="G11" t="n">
-        <v>45</v>
+        <v>82.17</v>
       </c>
       <c r="H11" t="n">
-        <v>30</v>
+        <v>65.89</v>
       </c>
       <c r="I11" t="n">
-        <v>15</v>
+        <v>16.28</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>373692</v>
+        <v>373648</v>
       </c>
       <c r="C12" t="n">
-        <v>54</v>
+        <v>142</v>
       </c>
       <c r="D12" t="n">
-        <v>20</v>
+        <v>111</v>
       </c>
       <c r="E12" t="n">
-        <v>18</v>
+        <v>87</v>
       </c>
       <c r="F12" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="G12" t="n">
-        <v>37.04</v>
+        <v>78.17</v>
       </c>
       <c r="H12" t="n">
-        <v>33.33</v>
+        <v>61.27</v>
       </c>
       <c r="I12" t="n">
-        <v>3.7</v>
+        <v>16.9</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Chashm Gul</t>
+          <t>Irum Ikram</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373695</v>
+        <v>373642</v>
       </c>
       <c r="C13" t="n">
-        <v>31</v>
+        <v>140</v>
       </c>
       <c r="D13" t="n">
-        <v>9</v>
+        <v>104</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="F13" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G13" t="n">
-        <v>29.03</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>69.29000000000001</v>
       </c>
       <c r="I13" t="n">
-        <v>29.03</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Summiya Hayat</t>
+          <t>Kainat</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>373710</v>
+        <v>373712</v>
       </c>
       <c r="C14" t="n">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="D14" t="n">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="E14" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F14" t="n">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="G14" t="n">
-        <v>25.93</v>
+        <v>73.33</v>
       </c>
       <c r="H14" t="n">
-        <v>12.35</v>
+        <v>21.67</v>
       </c>
       <c r="I14" t="n">
-        <v>13.58</v>
+        <v>51.67</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Muniba Shamim</t>
+          <t>Lati Khan</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373659</v>
+        <v>373665</v>
       </c>
       <c r="C15" t="n">
-        <v>72</v>
+        <v>45</v>
       </c>
       <c r="D15" t="n">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="F15" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="G15" t="n">
-        <v>25</v>
+        <v>71.11</v>
       </c>
       <c r="H15" t="n">
-        <v>2.78</v>
+        <v>64.44</v>
       </c>
       <c r="I15" t="n">
-        <v>22.22</v>
+        <v>6.67</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Naureen</t>
+          <t>Samara</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>884887</v>
+        <v>373658</v>
       </c>
       <c r="C16" t="n">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="D16" t="n">
-        <v>12</v>
+        <v>47</v>
       </c>
       <c r="E16" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F16" t="n">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="G16" t="n">
-        <v>23.53</v>
+        <v>64.38</v>
       </c>
       <c r="H16" t="n">
-        <v>19.61</v>
+        <v>15.07</v>
       </c>
       <c r="I16" t="n">
-        <v>3.92</v>
+        <v>49.32</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Rehana Bibi</t>
+          <t>Zohra</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>373691</v>
+        <v>373692</v>
       </c>
       <c r="C17" t="n">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D17" t="n">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="E17" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F17" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="G17" t="n">
-        <v>22.81</v>
+        <v>61.11</v>
       </c>
       <c r="H17" t="n">
-        <v>17.54</v>
+        <v>22.22</v>
       </c>
       <c r="I17" t="n">
-        <v>5.26</v>
+        <v>38.89</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Alia Khan</t>
+          <t>Muhammad Yousaf</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>373681</v>
+        <v>373690</v>
       </c>
       <c r="C18" t="n">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="D18" t="n">
-        <v>23</v>
+        <v>72</v>
       </c>
       <c r="E18" t="n">
-        <v>18</v>
+        <v>64</v>
       </c>
       <c r="F18" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G18" t="n">
-        <v>20.35</v>
+        <v>60.5</v>
       </c>
       <c r="H18" t="n">
-        <v>15.93</v>
+        <v>53.78</v>
       </c>
       <c r="I18" t="n">
-        <v>4.42</v>
+        <v>6.72</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Rehana Bibi</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>373648</v>
+        <v>373691</v>
       </c>
       <c r="C19" t="n">
-        <v>142</v>
+        <v>57</v>
       </c>
       <c r="D19" t="n">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F19" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G19" t="n">
-        <v>16.9</v>
+        <v>59.65</v>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>12.28</v>
       </c>
       <c r="I19" t="n">
-        <v>16.9</v>
+        <v>47.37</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Asma Bibi</t>
+          <t>Naureen</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>373641</v>
+        <v>884887</v>
       </c>
       <c r="C20" t="n">
-        <v>129</v>
+        <v>51</v>
       </c>
       <c r="D20" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="F20" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="G20" t="n">
-        <v>15.5</v>
+        <v>58.82</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>54.9</v>
       </c>
       <c r="I20" t="n">
-        <v>15.5</v>
+        <v>3.92</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Mahnoorr</t>
+          <t>Javairia</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>373670</v>
+        <v>373651</v>
       </c>
       <c r="C21" t="n">
-        <v>13</v>
+        <v>68</v>
       </c>
       <c r="D21" t="n">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="F21" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G21" t="n">
-        <v>15.38</v>
+        <v>57.35</v>
       </c>
       <c r="H21" t="n">
-        <v>7.69</v>
+        <v>48.53</v>
       </c>
       <c r="I21" t="n">
-        <v>7.69</v>
+        <v>8.82</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Shazia begum</t>
+          <t>Muniba Shamim</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>373696</v>
+        <v>373659</v>
       </c>
       <c r="C22" t="n">
-        <v>141</v>
+        <v>72</v>
       </c>
       <c r="D22" t="n">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="E22" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="F22" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G22" t="n">
-        <v>14.89</v>
+        <v>55.56</v>
       </c>
       <c r="H22" t="n">
-        <v>0.71</v>
+        <v>30.56</v>
       </c>
       <c r="I22" t="n">
-        <v>14.18</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sadia Rustum</t>
+          <t>Mahnoor</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>373649</v>
+        <v>373705</v>
       </c>
       <c r="C23" t="n">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="D23" t="n">
-        <v>15</v>
+        <v>51</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="F23" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="G23" t="n">
-        <v>14.56</v>
+        <v>54.26</v>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="I23" t="n">
-        <v>14.56</v>
+        <v>4.26</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Sidra Khan</t>
+          <t>Summiya Hayat</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>373645</v>
+        <v>373710</v>
       </c>
       <c r="C24" t="n">
-        <v>7</v>
+        <v>81</v>
       </c>
       <c r="D24" t="n">
-        <v>1</v>
+        <v>41</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="F24" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="G24" t="n">
-        <v>14.29</v>
+        <v>50.62</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>34.57</v>
       </c>
       <c r="I24" t="n">
-        <v>14.29</v>
+        <v>16.05</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Javairia</t>
+          <t>Muhammad Naeem</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>373651</v>
+        <v>373694</v>
       </c>
       <c r="C25" t="n">
-        <v>68</v>
+        <v>6</v>
       </c>
       <c r="D25" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E25" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G25" t="n">
-        <v>13.24</v>
+        <v>50</v>
       </c>
       <c r="H25" t="n">
-        <v>5.88</v>
+        <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>7.35</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Muhammad Noor</t>
+          <t>Shehla Noor</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>373701</v>
+        <v>373650</v>
       </c>
       <c r="C26" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G26" t="n">
-        <v>12.5</v>
+        <v>50</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>12.5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Lati Khan</t>
+          <t>Laiba Shams</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>564273</v>
+        <v>373706</v>
       </c>
       <c r="C27" t="n">
-        <v>9</v>
+        <v>93</v>
       </c>
       <c r="D27" t="n">
-        <v>1</v>
+        <v>42</v>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="F27" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G27" t="n">
-        <v>11.11</v>
+        <v>45.16</v>
       </c>
       <c r="H27" t="n">
-        <v>0</v>
+        <v>38.71</v>
       </c>
       <c r="I27" t="n">
-        <v>11.11</v>
+        <v>6.45</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Bushra Ayub</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>373646</v>
+        <v>373671</v>
       </c>
       <c r="C28" t="n">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D28" t="n">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="E28" t="n">
-        <v>4</v>
+        <v>46</v>
       </c>
       <c r="F28" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G28" t="n">
-        <v>9.52</v>
+        <v>41.13</v>
       </c>
       <c r="H28" t="n">
-        <v>3.17</v>
+        <v>37.1</v>
       </c>
       <c r="I28" t="n">
-        <v>6.35</v>
+        <v>4.03</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Laiba Shams</t>
+          <t>Asma Gull</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>373706</v>
+        <v>373672</v>
       </c>
       <c r="C29" t="n">
-        <v>93</v>
+        <v>129</v>
       </c>
       <c r="D29" t="n">
-        <v>7</v>
+        <v>53</v>
       </c>
       <c r="E29" t="n">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="F29" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G29" t="n">
-        <v>7.53</v>
+        <v>41.09</v>
       </c>
       <c r="H29" t="n">
-        <v>1.08</v>
+        <v>34.88</v>
       </c>
       <c r="I29" t="n">
-        <v>6.45</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="30">
@@ -2220,562 +2296,562 @@
         <v>135</v>
       </c>
       <c r="D30" t="n">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="E30" t="n">
-        <v>2</v>
+        <v>46</v>
       </c>
       <c r="F30" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G30" t="n">
-        <v>7.41</v>
+        <v>40.74</v>
       </c>
       <c r="H30" t="n">
-        <v>1.48</v>
+        <v>34.07</v>
       </c>
       <c r="I30" t="n">
-        <v>5.93</v>
+        <v>6.67</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Asma Gull</t>
+          <t>Munawar Khan</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>373672</v>
+        <v>373668</v>
       </c>
       <c r="C31" t="n">
-        <v>129</v>
+        <v>63</v>
       </c>
       <c r="D31" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="E31" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="F31" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G31" t="n">
-        <v>6.98</v>
+        <v>39.68</v>
       </c>
       <c r="H31" t="n">
-        <v>1.55</v>
+        <v>31.75</v>
       </c>
       <c r="I31" t="n">
-        <v>5.43</v>
+        <v>7.94</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Lati Khan</t>
+          <t>Khalida Bibi</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>373665</v>
+        <v>373673</v>
       </c>
       <c r="C32" t="n">
-        <v>45</v>
+        <v>132</v>
       </c>
       <c r="D32" t="n">
-        <v>3</v>
+        <v>50</v>
       </c>
       <c r="E32" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="F32" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G32" t="n">
-        <v>6.67</v>
+        <v>37.88</v>
       </c>
       <c r="H32" t="n">
-        <v>0</v>
+        <v>34.85</v>
       </c>
       <c r="I32" t="n">
-        <v>6.67</v>
+        <v>3.03</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Muhammad Yousaf</t>
+          <t>Chashm Gul</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>373690</v>
+        <v>373695</v>
       </c>
       <c r="C33" t="n">
-        <v>119</v>
+        <v>31</v>
       </c>
       <c r="D33" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E33" t="n">
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G33" t="n">
-        <v>5.88</v>
+        <v>29.03</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>5.88</v>
+        <v>29.03</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Bushra Ayub</t>
+          <t>Muhammad Noor</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>373671</v>
+        <v>373701</v>
       </c>
       <c r="C34" t="n">
-        <v>124</v>
+        <v>8</v>
       </c>
       <c r="D34" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G34" t="n">
-        <v>5.65</v>
+        <v>25</v>
       </c>
       <c r="H34" t="n">
-        <v>1.61</v>
+        <v>12.5</v>
       </c>
       <c r="I34" t="n">
-        <v>4.03</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Anum Gul</t>
+          <t>Rahila Naaz</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>373656</v>
+        <v>373715</v>
       </c>
       <c r="C35" t="n">
-        <v>97</v>
+        <v>4</v>
       </c>
       <c r="D35" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G35" t="n">
-        <v>5.15</v>
+        <v>25</v>
       </c>
       <c r="H35" t="n">
         <v>0</v>
       </c>
       <c r="I35" t="n">
-        <v>5.15</v>
+        <v>25</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Zain Ul Abideen</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>373642</v>
+        <v>373667</v>
       </c>
       <c r="C36" t="n">
-        <v>140</v>
+        <v>13</v>
       </c>
       <c r="D36" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E36" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F36" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>5</v>
+        <v>23.08</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>23.08</v>
       </c>
       <c r="I36" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Mahnoor</t>
+          <t>Anum Gul</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>373705</v>
+        <v>373656</v>
       </c>
       <c r="C37" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D37" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="E37" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="F37" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G37" t="n">
-        <v>4.26</v>
+        <v>17.53</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>12.37</v>
       </c>
       <c r="I37" t="n">
-        <v>4.26</v>
+        <v>5.15</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Munawar Khan</t>
+          <t>Muhammad Shahid Khan</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>373668</v>
+        <v>373662</v>
       </c>
       <c r="C38" t="n">
-        <v>63</v>
+        <v>6</v>
       </c>
       <c r="D38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>3.17</v>
+        <v>16.67</v>
       </c>
       <c r="H38" t="n">
-        <v>0</v>
+        <v>16.67</v>
       </c>
       <c r="I38" t="n">
-        <v>3.17</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Khalida Bibi</t>
+          <t>Sidra Khan</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>373673</v>
+        <v>373645</v>
       </c>
       <c r="C39" t="n">
-        <v>132</v>
+        <v>7</v>
       </c>
       <c r="D39" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E39" t="n">
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G39" t="n">
-        <v>3.03</v>
+        <v>14.29</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
       </c>
       <c r="I39" t="n">
-        <v>3.03</v>
+        <v>14.29</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Ishaq Khan</t>
+          <t>Robina Shaheen</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>373699</v>
+        <v>373639</v>
       </c>
       <c r="C40" t="n">
-        <v>116</v>
+        <v>8</v>
       </c>
       <c r="D40" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E40" t="n">
         <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G40" t="n">
-        <v>2.59</v>
+        <v>12.5</v>
       </c>
       <c r="H40" t="n">
         <v>0</v>
       </c>
       <c r="I40" t="n">
-        <v>2.59</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Nillum Bibi</t>
+          <t>Alia Khan</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>373652</v>
+        <v>373681</v>
       </c>
       <c r="C41" t="n">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="D41" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E41" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F41" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G41" t="n">
-        <v>2.52</v>
+        <v>10.62</v>
       </c>
       <c r="H41" t="n">
-        <v>0</v>
+        <v>6.19</v>
       </c>
       <c r="I41" t="n">
-        <v>2.52</v>
+        <v>4.42</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Laiba Khan</t>
+          <t>Aisha Aman</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>373653</v>
+        <v>373704</v>
       </c>
       <c r="C42" t="n">
-        <v>104</v>
+        <v>11</v>
       </c>
       <c r="D42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F42" t="n">
         <v>1</v>
       </c>
       <c r="G42" t="n">
-        <v>1.92</v>
+        <v>9.09</v>
       </c>
       <c r="H42" t="n">
-        <v>0.96</v>
+        <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>0.96</v>
+        <v>9.09</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Jaweria</t>
+          <t>Laiba Khan</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>163495</v>
+        <v>373653</v>
       </c>
       <c r="C43" t="n">
-        <v>68</v>
+        <v>104</v>
       </c>
       <c r="D43" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E43" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F43" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G43" t="n">
-        <v>1.47</v>
+        <v>7.69</v>
       </c>
       <c r="H43" t="n">
-        <v>0</v>
+        <v>3.85</v>
       </c>
       <c r="I43" t="n">
-        <v>1.47</v>
+        <v>3.85</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Aisha Aman</t>
+          <t>Mahnoorr</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>373704</v>
+        <v>373670</v>
       </c>
       <c r="C44" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E44" t="n">
         <v>0</v>
       </c>
       <c r="F44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G44" t="n">
-        <v>0</v>
+        <v>7.69</v>
       </c>
       <c r="H44" t="n">
         <v>0</v>
       </c>
       <c r="I44" t="n">
-        <v>0</v>
+        <v>7.69</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Gul Rukh</t>
+          <t>Ishaq Khan</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>373644</v>
+        <v>373699</v>
       </c>
       <c r="C45" t="n">
-        <v>6</v>
+        <v>116</v>
       </c>
       <c r="D45" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E45" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F45" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G45" t="n">
-        <v>0</v>
+        <v>6.9</v>
       </c>
       <c r="H45" t="n">
-        <v>0</v>
+        <v>4.31</v>
       </c>
       <c r="I45" t="n">
-        <v>0</v>
+        <v>2.59</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Iqra Bibi</t>
+          <t>Nillum Bibi</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>373708</v>
+        <v>373652</v>
       </c>
       <c r="C46" t="n">
+        <v>119</v>
+      </c>
+      <c r="D46" t="n">
         <v>8</v>
       </c>
-      <c r="D46" t="n">
-        <v>0</v>
-      </c>
       <c r="E46" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F46" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G46" t="n">
-        <v>0</v>
+        <v>6.72</v>
       </c>
       <c r="H46" t="n">
-        <v>0</v>
+        <v>2.52</v>
       </c>
       <c r="I46" t="n">
-        <v>0</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Irum ikram</t>
+          <t>Nazia</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>541376</v>
+        <v>373657</v>
       </c>
       <c r="C47" t="n">
-        <v>8</v>
+        <v>97</v>
       </c>
       <c r="D47" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E47" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G47" t="n">
-        <v>0</v>
+        <v>5.15</v>
       </c>
       <c r="H47" t="n">
-        <v>0</v>
+        <v>4.12</v>
       </c>
       <c r="I47" t="n">
-        <v>0</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Lati Khan (duplicate name received from listed_girl_tracking_survey on June 28, 2026 10:43 UTC+00:00; submission key: uuid:e4e89d53-e5be-40ff-bb2c-fa94c0d50011)</t>
+          <t>Gul Rukh</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>564273</v>
+        <v>373644</v>
       </c>
       <c r="C48" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="D48" t="n">
         <v>0</v>
@@ -2799,14 +2875,14 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Lati khan</t>
+          <t>Hijab Zahra</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>652938</v>
+        <v>373637</v>
       </c>
       <c r="C49" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D49" t="n">
         <v>0</v>
@@ -2830,14 +2906,14 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Lati khan</t>
+          <t>Iqra Bibi</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>671211</v>
+        <v>373708</v>
       </c>
       <c r="C50" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D50" t="n">
         <v>0</v>
@@ -2861,14 +2937,14 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Lati khan (duplicate name received from listed_girl_tracking_survey_new_sample on July 4, 2026 14:31 UTC+00:00; submission key: uuid:6316d214-c458-4786-937a-bd81b08c15c5)</t>
+          <t>Irum ikram</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>671211</v>
+        <v>541376</v>
       </c>
       <c r="C51" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="D51" t="n">
         <v>0</v>
@@ -2892,14 +2968,14 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Muhammad Shahid Khan</t>
+          <t>Lati Khan (duplicate name received from listed_girl_tracking_survey on June 28, 2026 10:43 UTC+00:00; submission key: uuid:e4e89d53-e5be-40ff-bb2c-fa94c0d50011)</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>373662</v>
+        <v>564273</v>
       </c>
       <c r="C52" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="D52" t="n">
         <v>0</v>
@@ -2923,14 +2999,14 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Muhammad Usman</t>
+          <t>Lati khan</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>373666</v>
+        <v>652938</v>
       </c>
       <c r="C53" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D53" t="n">
         <v>0</v>
@@ -2954,14 +3030,14 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Muhammad Waseem</t>
+          <t>Lati khan (duplicate name received from listed_girl_tracking_survey_new_sample on July 4, 2026 14:31 UTC+00:00; submission key: uuid:6316d214-c458-4786-937a-bd81b08c15c5)</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>373689</v>
+        <v>671211</v>
       </c>
       <c r="C54" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="D54" t="n">
         <v>0</v>
@@ -2985,14 +3061,14 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Muhammad naeem (duplicate name received from primary_school_listing_survey on February 14, 2026 14:38 UTC+00:00; submission key: uuid:5f0e427e-5fd2-4474-be64-ae5f2c4617a2)</t>
+          <t>Muhammad Usman</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>571571</v>
+        <v>373666</v>
       </c>
       <c r="C55" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="D55" t="n">
         <v>0</v>
@@ -3016,14 +3092,14 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Nadia bibi</t>
+          <t>Muhammad Waseem</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>373669</v>
+        <v>373689</v>
       </c>
       <c r="C56" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D56" t="n">
         <v>0</v>
@@ -3047,14 +3123,14 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Naureen Khan</t>
+          <t>Muhammad naeem (duplicate name received from primary_school_listing_survey on February 14, 2026 14:38 UTC+00:00; submission key: uuid:5f0e427e-5fd2-4474-be64-ae5f2c4617a2)</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>373716</v>
+        <v>571571</v>
       </c>
       <c r="C57" t="n">
-        <v>53</v>
+        <v>8</v>
       </c>
       <c r="D57" t="n">
         <v>0</v>
@@ -3078,14 +3154,14 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Naureen khan</t>
+          <t>Nadia bibi</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>453925</v>
+        <v>373669</v>
       </c>
       <c r="C58" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D58" t="n">
         <v>0</v>
@@ -3140,14 +3216,14 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Nazia</t>
+          <t>Saba Ramzan</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>373657</v>
+        <v>373703</v>
       </c>
       <c r="C60" t="n">
-        <v>97</v>
+        <v>13</v>
       </c>
       <c r="D60" t="n">
         <v>0</v>
@@ -3171,14 +3247,14 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Rahila Naaz</t>
+          <t>Sadia rustum</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>373715</v>
+        <v>852541</v>
       </c>
       <c r="C61" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D61" t="n">
         <v>0</v>
@@ -3202,11 +3278,11 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Robina Shaheen</t>
+          <t>Sajjad Khan</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>373639</v>
+        <v>373700</v>
       </c>
       <c r="C62" t="n">
         <v>8</v>
@@ -3233,14 +3309,14 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Saba Ramzan</t>
+          <t>Samreen</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>373703</v>
+        <v>373711</v>
       </c>
       <c r="C63" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="D63" t="n">
         <v>0</v>
@@ -3264,14 +3340,14 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Sadia rustum</t>
+          <t>Samreen</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>852541</v>
+        <v>639258</v>
       </c>
       <c r="C64" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D64" t="n">
         <v>0</v>
@@ -3295,11 +3371,11 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Samreen</t>
+          <t>Shakeel Ahmed</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>373711</v>
+        <v>373686</v>
       </c>
       <c r="C65" t="n">
         <v>3</v>
@@ -3326,14 +3402,14 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Shakeel Ahmed</t>
+          <t>Syed Haider Abbas</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>373686</v>
+        <v>373713</v>
       </c>
       <c r="C66" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D66" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Enhance duration handling and duplicate record checks in survey scripts
- Introduced a preference for SurveyCTO duration in the girls and household scripts, allowing for more accurate survey duration calculations.
- Added functions to retain recommendations for handling duplicate records, improving the clarity of issues flagged during data validation.
- Updated error guidance to reflect new checks for identity mismatches and duplicate records across household and girls surveys.
- Adjusted configuration files to set default values for critical fast duration and minimum survey duration, enhancing data integrity checks.
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -920,96 +920,96 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Naureen khan</t>
+          <t>Samara</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>453925</v>
+        <v>373658</v>
       </c>
       <c r="C27" t="n">
-        <v>18</v>
+        <v>59</v>
       </c>
       <c r="D27" t="n">
         <v>18</v>
       </c>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Kainat</t>
+          <t>Naureen khan</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>373712</v>
+        <v>453925</v>
       </c>
       <c r="C28" t="n">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="D28" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E28" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Kainat</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>373692</v>
+        <v>373712</v>
       </c>
       <c r="C29" t="n">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="D29" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E29" t="n">
-        <v>21</v>
+        <v>36</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Anum Gul</t>
+          <t>Zohra</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>373656</v>
+        <v>373692</v>
       </c>
       <c r="C30" t="n">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="D30" t="n">
         <v>12</v>
       </c>
       <c r="E30" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Samara</t>
+          <t>Anum Gul</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>373658</v>
+        <v>373656</v>
       </c>
       <c r="C31" t="n">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="D31" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E31" t="n">
-        <v>36</v>
+        <v>5</v>
       </c>
     </row>
     <row r="32">
@@ -1022,13 +1022,13 @@
         <v>373691</v>
       </c>
       <c r="C32" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D32" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E32" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="33">
@@ -1573,404 +1573,404 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Shazia begum</t>
+          <t>Kainat</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>373696</v>
+        <v>373712</v>
       </c>
       <c r="C7" t="n">
-        <v>141</v>
+        <v>60</v>
       </c>
       <c r="D7" t="n">
-        <v>120</v>
+        <v>53</v>
       </c>
       <c r="E7" t="n">
-        <v>100</v>
+        <v>17</v>
       </c>
       <c r="F7" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="G7" t="n">
-        <v>85.11</v>
+        <v>88.33</v>
       </c>
       <c r="H7" t="n">
-        <v>70.92</v>
+        <v>28.33</v>
       </c>
       <c r="I7" t="n">
-        <v>14.18</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Sadia Rustum</t>
+          <t>Shazia begum</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>373649</v>
+        <v>373696</v>
       </c>
       <c r="C8" t="n">
-        <v>103</v>
+        <v>141</v>
       </c>
       <c r="D8" t="n">
-        <v>87</v>
+        <v>120</v>
       </c>
       <c r="E8" t="n">
-        <v>72</v>
+        <v>100</v>
       </c>
       <c r="F8" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G8" t="n">
-        <v>84.47</v>
+        <v>85.11</v>
       </c>
       <c r="H8" t="n">
-        <v>69.90000000000001</v>
+        <v>70.92</v>
       </c>
       <c r="I8" t="n">
-        <v>14.56</v>
+        <v>14.18</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Jaweria</t>
+          <t>Sadia Rustum</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>163495</v>
+        <v>373649</v>
       </c>
       <c r="C9" t="n">
-        <v>68</v>
+        <v>103</v>
       </c>
       <c r="D9" t="n">
-        <v>57</v>
+        <v>87</v>
       </c>
       <c r="E9" t="n">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="G9" t="n">
-        <v>83.81999999999999</v>
+        <v>84.47</v>
       </c>
       <c r="H9" t="n">
-        <v>82.34999999999999</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="I9" t="n">
-        <v>1.47</v>
+        <v>14.56</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Jaweria</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>373646</v>
+        <v>163495</v>
       </c>
       <c r="C10" t="n">
-        <v>126</v>
+        <v>68</v>
       </c>
       <c r="D10" t="n">
-        <v>104</v>
+        <v>57</v>
       </c>
       <c r="E10" t="n">
-        <v>96</v>
+        <v>56</v>
       </c>
       <c r="F10" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>82.54000000000001</v>
+        <v>83.81999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>76.19</v>
+        <v>82.34999999999999</v>
       </c>
       <c r="I10" t="n">
-        <v>6.35</v>
+        <v>1.47</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Asma Bibi</t>
+          <t>Shafaq Zahra</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>373641</v>
+        <v>373646</v>
       </c>
       <c r="C11" t="n">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D11" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E11" t="n">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="F11" t="n">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="G11" t="n">
-        <v>82.17</v>
+        <v>82.54000000000001</v>
       </c>
       <c r="H11" t="n">
-        <v>65.89</v>
+        <v>76.19</v>
       </c>
       <c r="I11" t="n">
-        <v>16.28</v>
+        <v>6.35</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Asma Bibi</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>373648</v>
+        <v>373641</v>
       </c>
       <c r="C12" t="n">
-        <v>142</v>
+        <v>129</v>
       </c>
       <c r="D12" t="n">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="E12" t="n">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F12" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="G12" t="n">
-        <v>78.17</v>
+        <v>82.17</v>
       </c>
       <c r="H12" t="n">
-        <v>61.27</v>
+        <v>65.89</v>
       </c>
       <c r="I12" t="n">
-        <v>16.9</v>
+        <v>16.28</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Samara</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373642</v>
+        <v>373658</v>
       </c>
       <c r="C13" t="n">
-        <v>140</v>
+        <v>73</v>
       </c>
       <c r="D13" t="n">
-        <v>104</v>
+        <v>59</v>
       </c>
       <c r="E13" t="n">
-        <v>97</v>
+        <v>18</v>
       </c>
       <c r="F13" t="n">
-        <v>7</v>
+        <v>41</v>
       </c>
       <c r="G13" t="n">
-        <v>74.29000000000001</v>
+        <v>80.81999999999999</v>
       </c>
       <c r="H13" t="n">
-        <v>69.29000000000001</v>
+        <v>24.66</v>
       </c>
       <c r="I13" t="n">
-        <v>5</v>
+        <v>56.16</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Kainat</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>373712</v>
+        <v>373648</v>
       </c>
       <c r="C14" t="n">
-        <v>60</v>
+        <v>142</v>
       </c>
       <c r="D14" t="n">
-        <v>44</v>
+        <v>111</v>
       </c>
       <c r="E14" t="n">
-        <v>13</v>
+        <v>87</v>
       </c>
       <c r="F14" t="n">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="G14" t="n">
-        <v>73.33</v>
+        <v>78.17</v>
       </c>
       <c r="H14" t="n">
-        <v>21.67</v>
+        <v>61.27</v>
       </c>
       <c r="I14" t="n">
-        <v>51.67</v>
+        <v>16.9</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Lati Khan</t>
+          <t>Irum Ikram</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373665</v>
+        <v>373642</v>
       </c>
       <c r="C15" t="n">
-        <v>45</v>
+        <v>140</v>
       </c>
       <c r="D15" t="n">
-        <v>32</v>
+        <v>104</v>
       </c>
       <c r="E15" t="n">
-        <v>29</v>
+        <v>97</v>
       </c>
       <c r="F15" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G15" t="n">
-        <v>71.11</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="H15" t="n">
-        <v>64.44</v>
+        <v>69.29000000000001</v>
       </c>
       <c r="I15" t="n">
-        <v>6.67</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Samara</t>
+          <t>Lati Khan</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>373658</v>
+        <v>373665</v>
       </c>
       <c r="C16" t="n">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="D16" t="n">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="E16" t="n">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="F16" t="n">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="G16" t="n">
-        <v>64.38</v>
+        <v>71.11</v>
       </c>
       <c r="H16" t="n">
-        <v>15.07</v>
+        <v>64.44</v>
       </c>
       <c r="I16" t="n">
-        <v>49.32</v>
+        <v>6.67</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Rehana Bibi</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>373692</v>
+        <v>373691</v>
       </c>
       <c r="C17" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D17" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="E17" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F17" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="G17" t="n">
-        <v>61.11</v>
+        <v>66.67</v>
       </c>
       <c r="H17" t="n">
-        <v>22.22</v>
+        <v>14.04</v>
       </c>
       <c r="I17" t="n">
-        <v>38.89</v>
+        <v>52.63</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Muhammad Yousaf</t>
+          <t>Zohra</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>373690</v>
+        <v>373692</v>
       </c>
       <c r="C18" t="n">
-        <v>119</v>
+        <v>54</v>
       </c>
       <c r="D18" t="n">
-        <v>72</v>
+        <v>33</v>
       </c>
       <c r="E18" t="n">
-        <v>64</v>
+        <v>12</v>
       </c>
       <c r="F18" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="G18" t="n">
-        <v>60.5</v>
+        <v>61.11</v>
       </c>
       <c r="H18" t="n">
-        <v>53.78</v>
+        <v>22.22</v>
       </c>
       <c r="I18" t="n">
-        <v>6.72</v>
+        <v>38.89</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Rehana Bibi</t>
+          <t>Muhammad Yousaf</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>373691</v>
+        <v>373690</v>
       </c>
       <c r="C19" t="n">
-        <v>57</v>
+        <v>119</v>
       </c>
       <c r="D19" t="n">
-        <v>34</v>
+        <v>72</v>
       </c>
       <c r="E19" t="n">
-        <v>7</v>
+        <v>64</v>
       </c>
       <c r="F19" t="n">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="G19" t="n">
-        <v>59.65</v>
+        <v>60.5</v>
       </c>
       <c r="H19" t="n">
-        <v>12.28</v>
+        <v>53.78</v>
       </c>
       <c r="I19" t="n">
-        <v>47.37</v>
+        <v>6.72</v>
       </c>
     </row>
     <row r="20">

</xml_diff>

<commit_message>
Update error log files to reflect recent changes in data handling
- Modified the Daily Error Log, Enumerator Performance, and Weekly QA Summary Excel files to incorporate the latest error reporting standards and data integrity improvements.
- Ensured consistency across error logs following recent updates to error handling protocols.
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,10 +452,10 @@
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
-        <v>2102</v>
+        <v>2250</v>
       </c>
       <c r="D2" t="n">
-        <v>2102</v>
+        <v>2250</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -471,51 +471,51 @@
         <v>373696</v>
       </c>
       <c r="C3" t="n">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D3" t="n">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="E3" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Shafaq Zahra</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>373642</v>
+        <v>373646</v>
       </c>
       <c r="C4" t="n">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="D4" t="n">
-        <v>97</v>
+        <v>107</v>
       </c>
       <c r="E4" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Irum Ikram</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>373646</v>
+        <v>373642</v>
       </c>
       <c r="C5" t="n">
+        <v>108</v>
+      </c>
+      <c r="D5" t="n">
         <v>104</v>
       </c>
-      <c r="D5" t="n">
-        <v>96</v>
-      </c>
       <c r="E5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -528,13 +528,13 @@
         <v>373648</v>
       </c>
       <c r="C6" t="n">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="D6" t="n">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="E6" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7">
@@ -547,51 +547,51 @@
         <v>373641</v>
       </c>
       <c r="C7" t="n">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="D7" t="n">
-        <v>85</v>
+        <v>99</v>
       </c>
       <c r="E7" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Mehran Khan</t>
+          <t>Sadia Rustum</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>373684</v>
+        <v>373649</v>
       </c>
       <c r="C8" t="n">
-        <v>178</v>
+        <v>92</v>
       </c>
       <c r="D8" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E8" t="n">
-        <v>99</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sadia Rustum</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>373649</v>
+        <v>373684</v>
       </c>
       <c r="C9" t="n">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="D9" t="n">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="E9" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10">
@@ -604,10 +604,10 @@
         <v>373690</v>
       </c>
       <c r="C10" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D10" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E10" t="n">
         <v>8</v>
@@ -623,10 +623,10 @@
         <v>163495</v>
       </c>
       <c r="C11" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D11" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E11" t="n">
         <v>1</v>
@@ -642,10 +642,10 @@
         <v>373716</v>
       </c>
       <c r="C12" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="D12" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
@@ -654,131 +654,131 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Mahnoor</t>
+          <t>Javairia</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373705</v>
+        <v>373651</v>
       </c>
       <c r="C13" t="n">
+        <v>62</v>
+      </c>
+      <c r="D13" t="n">
         <v>51</v>
       </c>
-      <c r="D13" t="n">
-        <v>47</v>
-      </c>
       <c r="E13" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Furqan Ullah Khan</t>
+          <t>Mahnoor</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>373683</v>
+        <v>373705</v>
       </c>
       <c r="C14" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D14" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E14" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Bushra Ayub</t>
+          <t>Furqan Ullah Khan</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373671</v>
+        <v>373683</v>
       </c>
       <c r="C15" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D15" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Khalida Bibi</t>
+          <t>Bushra Ayub</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>373673</v>
+        <v>373671</v>
       </c>
       <c r="C16" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D16" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E16" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Asma Gull</t>
+          <t>Khalida Bibi</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>373672</v>
+        <v>373673</v>
       </c>
       <c r="C17" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="D17" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E17" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Laiba Shams</t>
+          <t>Asma Gull</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>373706</v>
+        <v>373672</v>
       </c>
       <c r="C18" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D18" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="E18" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Javairia</t>
+          <t>Laiba Shams</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>373651</v>
+        <v>373706</v>
       </c>
       <c r="C19" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D19" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E19" t="n">
         <v>6</v>
@@ -794,162 +794,162 @@
         <v>373665</v>
       </c>
       <c r="C20" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D20" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Summiya Hayat</t>
+          <t>Naureen</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>373710</v>
+        <v>884887</v>
       </c>
       <c r="C21" t="n">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="D21" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E21" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Naureen</t>
+          <t>Lati Khan</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>884887</v>
+        <v>564273</v>
       </c>
       <c r="C22" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D22" t="n">
         <v>28</v>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Muniba Shamim</t>
+          <t>Summiya Hayat</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>373659</v>
+        <v>373710</v>
       </c>
       <c r="C23" t="n">
         <v>40</v>
       </c>
       <c r="D23" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="E23" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Munawar Khan</t>
+          <t>Naureen khan</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>373668</v>
+        <v>453925</v>
       </c>
       <c r="C24" t="n">
         <v>25</v>
       </c>
       <c r="D24" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E24" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Lati Khan</t>
+          <t>Muniba Shamim</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>564273</v>
+        <v>373659</v>
       </c>
       <c r="C25" t="n">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="D25" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E25" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Lati khan</t>
+          <t>Munawar Khan</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>671211</v>
+        <v>373668</v>
       </c>
       <c r="C26" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="D26" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Samara</t>
+          <t>Zohra</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>373658</v>
+        <v>373692</v>
       </c>
       <c r="C27" t="n">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D27" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E27" t="n">
-        <v>41</v>
+        <v>33</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Naureen khan</t>
+          <t>Lati khan</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>453925</v>
+        <v>671211</v>
       </c>
       <c r="C28" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D28" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
@@ -965,10 +965,10 @@
         <v>373712</v>
       </c>
       <c r="C29" t="n">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="D29" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E29" t="n">
         <v>36</v>
@@ -977,20 +977,20 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Samara</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>373692</v>
+        <v>373658</v>
       </c>
       <c r="C30" t="n">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="D30" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E30" t="n">
-        <v>21</v>
+        <v>34</v>
       </c>
     </row>
     <row r="31">
@@ -1006,10 +1006,10 @@
         <v>17</v>
       </c>
       <c r="D31" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E31" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="32">
@@ -1022,13 +1022,13 @@
         <v>373691</v>
       </c>
       <c r="C32" t="n">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="D32" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E32" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
     </row>
     <row r="33">
@@ -1041,29 +1041,29 @@
         <v>373681</v>
       </c>
       <c r="C33" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D33" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E33" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Ishaq Khan</t>
+          <t>Irum ikram</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>373699</v>
+        <v>541376</v>
       </c>
       <c r="C34" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D34" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E34" t="n">
         <v>3</v>
@@ -1072,96 +1072,96 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Laiba Khan</t>
+          <t>Ishaq Khan</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>373653</v>
+        <v>373699</v>
       </c>
       <c r="C35" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D35" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E35" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Nazia</t>
+          <t>Laiba Khan</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>373657</v>
+        <v>373653</v>
       </c>
       <c r="C36" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D36" t="n">
         <v>4</v>
       </c>
       <c r="E36" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Nillum Bibi</t>
+          <t>Nazia</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>373652</v>
+        <v>373657</v>
       </c>
       <c r="C37" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D37" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E37" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Zain Ul Abideen</t>
+          <t>Nillum Bibi</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>373667</v>
+        <v>373652</v>
       </c>
       <c r="C38" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D38" t="n">
         <v>3</v>
       </c>
       <c r="E38" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Muhammad Noor</t>
+          <t>Zain Ul Abideen</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>373701</v>
+        <v>373667</v>
       </c>
       <c r="C39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D39" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -1174,10 +1174,10 @@
         <v>373662</v>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E40" t="n">
         <v>0</v>
@@ -1212,61 +1212,61 @@
         <v>571571</v>
       </c>
       <c r="C42" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D42" t="n">
         <v>0</v>
       </c>
       <c r="E42" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Muhammad Naeem</t>
+          <t>Aisha Aman</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>373694</v>
+        <v>373704</v>
       </c>
       <c r="C43" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D43" t="n">
         <v>0</v>
       </c>
       <c r="E43" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Shehla Noor</t>
+          <t>Mahnoorr</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>373650</v>
+        <v>373670</v>
       </c>
       <c r="C44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D44" t="n">
         <v>0</v>
       </c>
       <c r="E44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Aisha Aman</t>
+          <t>Muhammad Noor</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>373704</v>
+        <v>373701</v>
       </c>
       <c r="C45" t="n">
         <v>1</v>
@@ -1281,11 +1281,11 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Mahnoorr</t>
+          <t>Rahila Naaz</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>373670</v>
+        <v>373715</v>
       </c>
       <c r="C46" t="n">
         <v>1</v>
@@ -1300,11 +1300,11 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Rahila Naaz</t>
+          <t>Robina Shaheen</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>373715</v>
+        <v>373639</v>
       </c>
       <c r="C47" t="n">
         <v>1</v>
@@ -1313,44 +1313,6 @@
         <v>0</v>
       </c>
       <c r="E47" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Robina Shaheen</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>373639</v>
-      </c>
-      <c r="C48" t="n">
-        <v>1</v>
-      </c>
-      <c r="D48" t="n">
-        <v>0</v>
-      </c>
-      <c r="E48" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Sidra Khan</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>373645</v>
-      </c>
-      <c r="C49" t="n">
-        <v>1</v>
-      </c>
-      <c r="D49" t="n">
-        <v>0</v>
-      </c>
-      <c r="E49" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1365,7 +1327,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I67"/>
+  <dimension ref="A1:I68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1428,19 +1390,19 @@
         <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="E2" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>900</v>
+        <v>1250</v>
       </c>
       <c r="H2" t="n">
-        <v>900</v>
+        <v>1250</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -1459,19 +1421,19 @@
         <v>9</v>
       </c>
       <c r="D3" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="E3" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="F3" t="n">
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>233.33</v>
+        <v>322.22</v>
       </c>
       <c r="H3" t="n">
-        <v>222.22</v>
+        <v>311.11</v>
       </c>
       <c r="I3" t="n">
         <v>11.11</v>
@@ -1511,156 +1473,156 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Mehran Khan</t>
+          <t>Irum ikram</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>373684</v>
+        <v>541376</v>
       </c>
       <c r="C5" t="n">
-        <v>134</v>
+        <v>8</v>
       </c>
       <c r="D5" t="n">
-        <v>178</v>
+        <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>79</v>
+        <v>7</v>
       </c>
       <c r="F5" t="n">
-        <v>99</v>
+        <v>3</v>
       </c>
       <c r="G5" t="n">
-        <v>132.84</v>
+        <v>125</v>
       </c>
       <c r="H5" t="n">
-        <v>58.96</v>
+        <v>87.5</v>
       </c>
       <c r="I5" t="n">
-        <v>73.88</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Naureen Khan</t>
+          <t>Kainat</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>373716</v>
+        <v>373712</v>
       </c>
       <c r="C6" t="n">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="D6" t="n">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="E6" t="n">
-        <v>48</v>
+        <v>14</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="G6" t="n">
-        <v>90.56999999999999</v>
+        <v>88.41</v>
       </c>
       <c r="H6" t="n">
-        <v>90.56999999999999</v>
+        <v>20.29</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>52.17</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Kainat</t>
+          <t>Naureen Khan</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>373712</v>
+        <v>373716</v>
       </c>
       <c r="C7" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D7" t="n">
         <v>53</v>
       </c>
       <c r="E7" t="n">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="F7" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>88.33</v>
+        <v>85.48</v>
       </c>
       <c r="H7" t="n">
-        <v>28.33</v>
+        <v>85.48</v>
       </c>
       <c r="I7" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Shazia begum</t>
+          <t>Zohra</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>373696</v>
+        <v>373692</v>
       </c>
       <c r="C8" t="n">
-        <v>141</v>
+        <v>65</v>
       </c>
       <c r="D8" t="n">
-        <v>120</v>
+        <v>55</v>
       </c>
       <c r="E8" t="n">
-        <v>100</v>
+        <v>19</v>
       </c>
       <c r="F8" t="n">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="G8" t="n">
-        <v>85.11</v>
+        <v>84.62</v>
       </c>
       <c r="H8" t="n">
-        <v>70.92</v>
+        <v>29.23</v>
       </c>
       <c r="I8" t="n">
-        <v>14.18</v>
+        <v>50.77</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sadia Rustum</t>
+          <t>Rehana Bibi</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>373649</v>
+        <v>373691</v>
       </c>
       <c r="C9" t="n">
-        <v>103</v>
+        <v>69</v>
       </c>
       <c r="D9" t="n">
-        <v>87</v>
+        <v>58</v>
       </c>
       <c r="E9" t="n">
-        <v>72</v>
+        <v>11</v>
       </c>
       <c r="F9" t="n">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="G9" t="n">
-        <v>84.47</v>
+        <v>84.06</v>
       </c>
       <c r="H9" t="n">
-        <v>69.90000000000001</v>
+        <v>15.94</v>
       </c>
       <c r="I9" t="n">
-        <v>14.56</v>
+        <v>52.17</v>
       </c>
     </row>
     <row r="10">
@@ -1676,19 +1638,19 @@
         <v>68</v>
       </c>
       <c r="D10" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E10" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F10" t="n">
         <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>83.81999999999999</v>
+        <v>82.34999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>82.34999999999999</v>
+        <v>80.88</v>
       </c>
       <c r="I10" t="n">
         <v>1.47</v>
@@ -1697,373 +1659,373 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Shazia begum</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>373646</v>
+        <v>373696</v>
       </c>
       <c r="C11" t="n">
+        <v>160</v>
+      </c>
+      <c r="D11" t="n">
         <v>126</v>
       </c>
-      <c r="D11" t="n">
-        <v>104</v>
-      </c>
       <c r="E11" t="n">
-        <v>96</v>
+        <v>112</v>
       </c>
       <c r="F11" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="G11" t="n">
-        <v>82.54000000000001</v>
+        <v>78.75</v>
       </c>
       <c r="H11" t="n">
-        <v>76.19</v>
+        <v>70</v>
       </c>
       <c r="I11" t="n">
-        <v>6.35</v>
+        <v>8.75</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Asma Bibi</t>
+          <t>Shafaq Zahra</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>373641</v>
+        <v>373646</v>
       </c>
       <c r="C12" t="n">
-        <v>129</v>
+        <v>153</v>
       </c>
       <c r="D12" t="n">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="E12" t="n">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="F12" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="G12" t="n">
-        <v>82.17</v>
+        <v>77.78</v>
       </c>
       <c r="H12" t="n">
-        <v>65.89</v>
+        <v>69.93000000000001</v>
       </c>
       <c r="I12" t="n">
-        <v>16.28</v>
+        <v>7.84</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Samara</t>
+          <t>Asma Bibi</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373658</v>
+        <v>373641</v>
       </c>
       <c r="C13" t="n">
-        <v>73</v>
+        <v>150</v>
       </c>
       <c r="D13" t="n">
-        <v>59</v>
+        <v>113</v>
       </c>
       <c r="E13" t="n">
-        <v>18</v>
+        <v>99</v>
       </c>
       <c r="F13" t="n">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="G13" t="n">
-        <v>80.81999999999999</v>
+        <v>75.33</v>
       </c>
       <c r="H13" t="n">
-        <v>24.66</v>
+        <v>66</v>
       </c>
       <c r="I13" t="n">
-        <v>56.16</v>
+        <v>9.33</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Samara</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>373648</v>
+        <v>373658</v>
       </c>
       <c r="C14" t="n">
-        <v>142</v>
+        <v>83</v>
       </c>
       <c r="D14" t="n">
-        <v>111</v>
+        <v>62</v>
       </c>
       <c r="E14" t="n">
-        <v>87</v>
+        <v>13</v>
       </c>
       <c r="F14" t="n">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="G14" t="n">
-        <v>78.17</v>
+        <v>74.7</v>
       </c>
       <c r="H14" t="n">
-        <v>61.27</v>
+        <v>15.66</v>
       </c>
       <c r="I14" t="n">
-        <v>16.9</v>
+        <v>40.96</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373642</v>
+        <v>373648</v>
       </c>
       <c r="C15" t="n">
-        <v>140</v>
+        <v>164</v>
       </c>
       <c r="D15" t="n">
-        <v>104</v>
+        <v>120</v>
       </c>
       <c r="E15" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="F15" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="G15" t="n">
-        <v>74.29000000000001</v>
+        <v>73.17</v>
       </c>
       <c r="H15" t="n">
-        <v>69.29000000000001</v>
+        <v>61.59</v>
       </c>
       <c r="I15" t="n">
-        <v>5</v>
+        <v>11.59</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Lati Khan</t>
+          <t>Irum Ikram</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>373665</v>
+        <v>373642</v>
       </c>
       <c r="C16" t="n">
-        <v>45</v>
+        <v>149</v>
       </c>
       <c r="D16" t="n">
-        <v>32</v>
+        <v>108</v>
       </c>
       <c r="E16" t="n">
-        <v>29</v>
+        <v>104</v>
       </c>
       <c r="F16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G16" t="n">
-        <v>71.11</v>
+        <v>72.48</v>
       </c>
       <c r="H16" t="n">
-        <v>64.44</v>
+        <v>69.8</v>
       </c>
       <c r="I16" t="n">
-        <v>6.67</v>
+        <v>2.68</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Rehana Bibi</t>
+          <t>Sadia Rustum</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>373691</v>
+        <v>373649</v>
       </c>
       <c r="C17" t="n">
-        <v>57</v>
+        <v>130</v>
       </c>
       <c r="D17" t="n">
-        <v>38</v>
+        <v>92</v>
       </c>
       <c r="E17" t="n">
-        <v>8</v>
+        <v>82</v>
       </c>
       <c r="F17" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="G17" t="n">
-        <v>66.67</v>
+        <v>70.77</v>
       </c>
       <c r="H17" t="n">
-        <v>14.04</v>
+        <v>63.08</v>
       </c>
       <c r="I17" t="n">
-        <v>52.63</v>
+        <v>7.69</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Lati Khan</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>373692</v>
+        <v>373665</v>
       </c>
       <c r="C18" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D18" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E18" t="n">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="F18" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="G18" t="n">
-        <v>61.11</v>
+        <v>67.31</v>
       </c>
       <c r="H18" t="n">
-        <v>22.22</v>
+        <v>65.38</v>
       </c>
       <c r="I18" t="n">
-        <v>38.89</v>
+        <v>1.92</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Muhammad Yousaf</t>
+          <t>Javairia</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>373690</v>
+        <v>373651</v>
       </c>
       <c r="C19" t="n">
-        <v>119</v>
+        <v>95</v>
       </c>
       <c r="D19" t="n">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="E19" t="n">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="F19" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G19" t="n">
-        <v>60.5</v>
+        <v>65.26000000000001</v>
       </c>
       <c r="H19" t="n">
-        <v>53.78</v>
+        <v>53.68</v>
       </c>
       <c r="I19" t="n">
-        <v>6.72</v>
+        <v>11.58</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Naureen</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>884887</v>
+        <v>373684</v>
       </c>
       <c r="C20" t="n">
-        <v>51</v>
+        <v>158</v>
       </c>
       <c r="D20" t="n">
-        <v>30</v>
+        <v>102</v>
       </c>
       <c r="E20" t="n">
-        <v>28</v>
+        <v>79</v>
       </c>
       <c r="F20" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="G20" t="n">
-        <v>58.82</v>
+        <v>64.56</v>
       </c>
       <c r="H20" t="n">
-        <v>54.9</v>
+        <v>50</v>
       </c>
       <c r="I20" t="n">
-        <v>3.92</v>
+        <v>14.56</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Javairia</t>
+          <t>Muhammad Yousaf</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>373651</v>
+        <v>373690</v>
       </c>
       <c r="C21" t="n">
-        <v>68</v>
+        <v>119</v>
       </c>
       <c r="D21" t="n">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="E21" t="n">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="F21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G21" t="n">
-        <v>57.35</v>
+        <v>58.82</v>
       </c>
       <c r="H21" t="n">
-        <v>48.53</v>
+        <v>52.1</v>
       </c>
       <c r="I21" t="n">
-        <v>8.82</v>
+        <v>6.72</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Muniba Shamim</t>
+          <t>Naureen</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>373659</v>
+        <v>884887</v>
       </c>
       <c r="C22" t="n">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="D22" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="E22" t="n">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="F22" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="G22" t="n">
-        <v>55.56</v>
+        <v>58.33</v>
       </c>
       <c r="H22" t="n">
-        <v>30.56</v>
+        <v>51.67</v>
       </c>
       <c r="I22" t="n">
-        <v>25</v>
+        <v>6.67</v>
       </c>
     </row>
     <row r="23">
@@ -2079,19 +2041,19 @@
         <v>94</v>
       </c>
       <c r="D23" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E23" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F23" t="n">
         <v>4</v>
       </c>
       <c r="G23" t="n">
-        <v>54.26</v>
+        <v>56.38</v>
       </c>
       <c r="H23" t="n">
-        <v>50</v>
+        <v>52.13</v>
       </c>
       <c r="I23" t="n">
         <v>4.26</v>
@@ -2110,19 +2072,19 @@
         <v>81</v>
       </c>
       <c r="D24" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E24" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F24" t="n">
         <v>13</v>
       </c>
       <c r="G24" t="n">
-        <v>50.62</v>
+        <v>49.38</v>
       </c>
       <c r="H24" t="n">
-        <v>34.57</v>
+        <v>33.33</v>
       </c>
       <c r="I24" t="n">
         <v>16.05</v>
@@ -2131,94 +2093,94 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Muhammad Naeem</t>
+          <t>Muniba Shamim</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>373694</v>
+        <v>373659</v>
       </c>
       <c r="C25" t="n">
-        <v>6</v>
+        <v>72</v>
       </c>
       <c r="D25" t="n">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="F25" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G25" t="n">
-        <v>50</v>
+        <v>44.44</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>31.94</v>
       </c>
       <c r="I25" t="n">
-        <v>50</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Shehla Noor</t>
+          <t>Laiba Shams</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>373650</v>
+        <v>373706</v>
       </c>
       <c r="C26" t="n">
-        <v>4</v>
+        <v>93</v>
       </c>
       <c r="D26" t="n">
-        <v>2</v>
+        <v>41</v>
       </c>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="F26" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G26" t="n">
-        <v>50</v>
+        <v>44.09</v>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
+        <v>37.63</v>
       </c>
       <c r="I26" t="n">
-        <v>50</v>
+        <v>6.45</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Laiba Shams</t>
+          <t>Munawar Khan</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>373706</v>
+        <v>373668</v>
       </c>
       <c r="C27" t="n">
-        <v>93</v>
+        <v>63</v>
       </c>
       <c r="D27" t="n">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="E27" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="F27" t="n">
         <v>6</v>
       </c>
       <c r="G27" t="n">
-        <v>45.16</v>
+        <v>41.27</v>
       </c>
       <c r="H27" t="n">
-        <v>38.71</v>
+        <v>31.75</v>
       </c>
       <c r="I27" t="n">
-        <v>6.45</v>
+        <v>9.52</v>
       </c>
     </row>
     <row r="28">
@@ -2234,146 +2196,146 @@
         <v>124</v>
       </c>
       <c r="D28" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E28" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F28" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G28" t="n">
-        <v>41.13</v>
+        <v>39.52</v>
       </c>
       <c r="H28" t="n">
-        <v>37.1</v>
+        <v>37.9</v>
       </c>
       <c r="I28" t="n">
-        <v>4.03</v>
+        <v>1.61</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Asma Gull</t>
+          <t>Furqan Ullah Khan</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>373672</v>
+        <v>373683</v>
       </c>
       <c r="C29" t="n">
-        <v>129</v>
+        <v>142</v>
       </c>
       <c r="D29" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E29" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F29" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G29" t="n">
-        <v>41.09</v>
+        <v>36.62</v>
       </c>
       <c r="H29" t="n">
-        <v>34.88</v>
+        <v>33.8</v>
       </c>
       <c r="I29" t="n">
-        <v>6.2</v>
+        <v>2.82</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Furqan Ullah Khan</t>
+          <t>Asma Gull</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>373683</v>
+        <v>373672</v>
       </c>
       <c r="C30" t="n">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="D30" t="n">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="E30" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F30" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>40.74</v>
+        <v>35.66</v>
       </c>
       <c r="H30" t="n">
-        <v>34.07</v>
+        <v>34.88</v>
       </c>
       <c r="I30" t="n">
-        <v>6.67</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Munawar Khan</t>
+          <t>Khalida Bibi</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>373668</v>
+        <v>373673</v>
       </c>
       <c r="C31" t="n">
-        <v>63</v>
+        <v>140</v>
       </c>
       <c r="D31" t="n">
-        <v>25</v>
+        <v>47</v>
       </c>
       <c r="E31" t="n">
-        <v>20</v>
+        <v>47</v>
       </c>
       <c r="F31" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>39.68</v>
+        <v>33.57</v>
       </c>
       <c r="H31" t="n">
-        <v>31.75</v>
+        <v>33.57</v>
       </c>
       <c r="I31" t="n">
-        <v>7.94</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Khalida Bibi</t>
+          <t>Muhammad Shahid Khan</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>373673</v>
+        <v>373662</v>
       </c>
       <c r="C32" t="n">
-        <v>132</v>
+        <v>6</v>
       </c>
       <c r="D32" t="n">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="E32" t="n">
-        <v>46</v>
+        <v>2</v>
       </c>
       <c r="F32" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>37.88</v>
+        <v>33.33</v>
       </c>
       <c r="H32" t="n">
-        <v>34.85</v>
+        <v>33.33</v>
       </c>
       <c r="I32" t="n">
-        <v>3.03</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -2410,20 +2372,20 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Muhammad Noor</t>
+          <t>Rahila Naaz</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>373701</v>
+        <v>373715</v>
       </c>
       <c r="C34" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F34" t="n">
         <v>1</v>
@@ -2432,178 +2394,178 @@
         <v>25</v>
       </c>
       <c r="H34" t="n">
-        <v>12.5</v>
+        <v>0</v>
       </c>
       <c r="I34" t="n">
-        <v>12.5</v>
+        <v>25</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Rahila Naaz</t>
+          <t>Zain Ul Abideen</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>373715</v>
+        <v>373667</v>
       </c>
       <c r="C35" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="D35" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E35" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G35" t="n">
-        <v>25</v>
+        <v>23.08</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>23.08</v>
       </c>
       <c r="I35" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Zain Ul Abideen</t>
+          <t>Anum Gul</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>373667</v>
+        <v>373656</v>
       </c>
       <c r="C36" t="n">
+        <v>97</v>
+      </c>
+      <c r="D36" t="n">
+        <v>17</v>
+      </c>
+      <c r="E36" t="n">
         <v>13</v>
       </c>
-      <c r="D36" t="n">
-        <v>3</v>
-      </c>
-      <c r="E36" t="n">
-        <v>3</v>
-      </c>
       <c r="F36" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G36" t="n">
-        <v>23.08</v>
+        <v>17.53</v>
       </c>
       <c r="H36" t="n">
-        <v>23.08</v>
+        <v>13.4</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>4.12</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Anum Gul</t>
+          <t>Muhammad Noor</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>373656</v>
+        <v>373701</v>
       </c>
       <c r="C37" t="n">
-        <v>97</v>
+        <v>8</v>
       </c>
       <c r="D37" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G37" t="n">
-        <v>17.53</v>
+        <v>12.5</v>
       </c>
       <c r="H37" t="n">
-        <v>12.37</v>
+        <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>5.15</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Muhammad Shahid Khan</t>
+          <t>Robina Shaheen</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>373662</v>
+        <v>373639</v>
       </c>
       <c r="C38" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D38" t="n">
         <v>1</v>
       </c>
       <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="n">
         <v>1</v>
       </c>
-      <c r="F38" t="n">
-        <v>0</v>
-      </c>
       <c r="G38" t="n">
-        <v>16.67</v>
+        <v>12.5</v>
       </c>
       <c r="H38" t="n">
-        <v>16.67</v>
+        <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Sidra Khan</t>
+          <t>Alia Khan</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>373645</v>
+        <v>373681</v>
       </c>
       <c r="C39" t="n">
-        <v>7</v>
+        <v>113</v>
       </c>
       <c r="D39" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E39" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F39" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G39" t="n">
-        <v>14.29</v>
+        <v>11.5</v>
       </c>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>7.96</v>
       </c>
       <c r="I39" t="n">
-        <v>14.29</v>
+        <v>3.54</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Robina Shaheen</t>
+          <t>Aisha Aman</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>373639</v>
+        <v>373704</v>
       </c>
       <c r="C40" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D40" t="n">
         <v>1</v>
@@ -2615,57 +2577,57 @@
         <v>1</v>
       </c>
       <c r="G40" t="n">
-        <v>12.5</v>
+        <v>9.09</v>
       </c>
       <c r="H40" t="n">
         <v>0</v>
       </c>
       <c r="I40" t="n">
-        <v>12.5</v>
+        <v>9.09</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Alia Khan</t>
+          <t>Laiba Khan</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>373681</v>
+        <v>373653</v>
       </c>
       <c r="C41" t="n">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="D41" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E41" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F41" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G41" t="n">
-        <v>10.62</v>
+        <v>7.69</v>
       </c>
       <c r="H41" t="n">
-        <v>6.19</v>
+        <v>3.85</v>
       </c>
       <c r="I41" t="n">
-        <v>4.42</v>
+        <v>3.85</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Aisha Aman</t>
+          <t>Mahnoorr</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>373704</v>
+        <v>373670</v>
       </c>
       <c r="C42" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D42" t="n">
         <v>1</v>
@@ -2677,75 +2639,75 @@
         <v>1</v>
       </c>
       <c r="G42" t="n">
-        <v>9.09</v>
+        <v>7.69</v>
       </c>
       <c r="H42" t="n">
         <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>9.09</v>
+        <v>7.69</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Laiba Khan</t>
+          <t>Nazia</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>373653</v>
+        <v>373657</v>
       </c>
       <c r="C43" t="n">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="D43" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E43" t="n">
         <v>4</v>
       </c>
       <c r="F43" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G43" t="n">
-        <v>7.69</v>
+        <v>5.15</v>
       </c>
       <c r="H43" t="n">
-        <v>3.85</v>
+        <v>4.12</v>
       </c>
       <c r="I43" t="n">
-        <v>3.85</v>
+        <v>1.03</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Mahnoorr</t>
+          <t>Nillum Bibi</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>373670</v>
+        <v>373652</v>
       </c>
       <c r="C44" t="n">
-        <v>13</v>
+        <v>119</v>
       </c>
       <c r="D44" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E44" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F44" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G44" t="n">
-        <v>7.69</v>
+        <v>5.04</v>
       </c>
       <c r="H44" t="n">
-        <v>0</v>
+        <v>2.52</v>
       </c>
       <c r="I44" t="n">
-        <v>7.69</v>
+        <v>2.52</v>
       </c>
     </row>
     <row r="45">
@@ -2758,100 +2720,100 @@
         <v>373699</v>
       </c>
       <c r="C45" t="n">
-        <v>116</v>
+        <v>133</v>
       </c>
       <c r="D45" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E45" t="n">
         <v>5</v>
       </c>
       <c r="F45" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G45" t="n">
-        <v>6.9</v>
+        <v>4.51</v>
       </c>
       <c r="H45" t="n">
-        <v>4.31</v>
+        <v>3.76</v>
       </c>
       <c r="I45" t="n">
-        <v>2.59</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Nillum Bibi</t>
+          <t>Gul Rukh</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>373652</v>
+        <v>373644</v>
       </c>
       <c r="C46" t="n">
-        <v>119</v>
+        <v>6</v>
       </c>
       <c r="D46" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E46" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G46" t="n">
-        <v>6.72</v>
+        <v>0</v>
       </c>
       <c r="H46" t="n">
-        <v>2.52</v>
+        <v>0</v>
       </c>
       <c r="I46" t="n">
-        <v>4.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Nazia</t>
+          <t>Hijab Zahra</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>373657</v>
+        <v>373637</v>
       </c>
       <c r="C47" t="n">
-        <v>97</v>
+        <v>4</v>
       </c>
       <c r="D47" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E47" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G47" t="n">
-        <v>5.15</v>
+        <v>0</v>
       </c>
       <c r="H47" t="n">
-        <v>4.12</v>
+        <v>0</v>
       </c>
       <c r="I47" t="n">
-        <v>1.03</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Gul Rukh</t>
+          <t>Iqra Bibi</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>373644</v>
+        <v>373708</v>
       </c>
       <c r="C48" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D48" t="n">
         <v>0</v>
@@ -2875,14 +2837,14 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Hijab Zahra</t>
+          <t>Irum ikram (duplicate name received from listed_girl_tracking_survey on June 29, 2026 12:08 UTC+00:00; submission key: uuid:b700a976-75ee-467c-87e9-1d5163ec238d)</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>373637</v>
+        <v>541376</v>
       </c>
       <c r="C49" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="D49" t="n">
         <v>0</v>
@@ -2906,14 +2868,14 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Iqra Bibi</t>
+          <t>Lati Khan (duplicate name received from listed_girl_tracking_survey on June 28, 2026 10:43 UTC+00:00; submission key: uuid:e4e89d53-e5be-40ff-bb2c-fa94c0d50011)</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>373708</v>
+        <v>564273</v>
       </c>
       <c r="C50" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="D50" t="n">
         <v>0</v>
@@ -2937,14 +2899,14 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Irum ikram</t>
+          <t>Lati khan</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>541376</v>
+        <v>652938</v>
       </c>
       <c r="C51" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D51" t="n">
         <v>0</v>
@@ -2968,14 +2930,14 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Lati Khan (duplicate name received from listed_girl_tracking_survey on June 28, 2026 10:43 UTC+00:00; submission key: uuid:e4e89d53-e5be-40ff-bb2c-fa94c0d50011)</t>
+          <t>Lati khan (duplicate name received from listed_girl_tracking_survey_new_sample on July 4, 2026 14:31 UTC+00:00; submission key: uuid:6316d214-c458-4786-937a-bd81b08c15c5)</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>564273</v>
+        <v>671211</v>
       </c>
       <c r="C52" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="D52" t="n">
         <v>0</v>
@@ -2999,14 +2961,14 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Lati khan</t>
+          <t>Muhammad Naeem</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>652938</v>
+        <v>373694</v>
       </c>
       <c r="C53" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D53" t="n">
         <v>0</v>
@@ -3030,11 +2992,11 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Lati khan (duplicate name received from listed_girl_tracking_survey_new_sample on July 4, 2026 14:31 UTC+00:00; submission key: uuid:6316d214-c458-4786-937a-bd81b08c15c5)</t>
+          <t>Muhammad Usman</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>671211</v>
+        <v>373666</v>
       </c>
       <c r="C54" t="n">
         <v>14</v>
@@ -3061,14 +3023,14 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Muhammad Usman</t>
+          <t>Muhammad Waseem</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>373666</v>
+        <v>373689</v>
       </c>
       <c r="C55" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="D55" t="n">
         <v>0</v>
@@ -3092,14 +3054,14 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Muhammad Waseem</t>
+          <t>Muhammad naeem (duplicate name received from primary_school_listing_survey on February 14, 2026 14:38 UTC+00:00; submission key: uuid:5f0e427e-5fd2-4474-be64-ae5f2c4617a2)</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>373689</v>
+        <v>571571</v>
       </c>
       <c r="C56" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D56" t="n">
         <v>0</v>
@@ -3123,14 +3085,14 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Muhammad naeem (duplicate name received from primary_school_listing_survey on February 14, 2026 14:38 UTC+00:00; submission key: uuid:5f0e427e-5fd2-4474-be64-ae5f2c4617a2)</t>
+          <t>Nadia bibi</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>571571</v>
+        <v>373669</v>
       </c>
       <c r="C57" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D57" t="n">
         <v>0</v>
@@ -3154,14 +3116,14 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Nadia bibi</t>
+          <t>Naureen khan (duplicate name received from listed_girl_tracking_survey_new_sample on July 7, 2026 14:41 UTC+00:00; submission key: uuid:bbf56e1f-36f5-4ebf-9e0f-df83015a0871)</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>373669</v>
+        <v>453925</v>
       </c>
       <c r="C58" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="D58" t="n">
         <v>0</v>
@@ -3185,14 +3147,14 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Naureen khan (duplicate name received from listed_girl_tracking_survey_new_sample on July 7, 2026 14:41 UTC+00:00; submission key: uuid:bbf56e1f-36f5-4ebf-9e0f-df83015a0871)</t>
+          <t>Saba Ramzan</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>453925</v>
+        <v>373703</v>
       </c>
       <c r="C59" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D59" t="n">
         <v>0</v>
@@ -3216,14 +3178,14 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Saba Ramzan</t>
+          <t>Sadia rustum</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>373703</v>
+        <v>852541</v>
       </c>
       <c r="C60" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D60" t="n">
         <v>0</v>
@@ -3247,14 +3209,14 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Sadia rustum</t>
+          <t>Sajjad Khan</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>852541</v>
+        <v>373700</v>
       </c>
       <c r="C61" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D61" t="n">
         <v>0</v>
@@ -3278,14 +3240,14 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Sajjad Khan</t>
+          <t>Samreen</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>373700</v>
+        <v>373711</v>
       </c>
       <c r="C62" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D62" t="n">
         <v>0</v>
@@ -3313,10 +3275,10 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>373711</v>
+        <v>639258</v>
       </c>
       <c r="C63" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D63" t="n">
         <v>0</v>
@@ -3340,14 +3302,14 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Samreen</t>
+          <t>Shakeel Ahmed</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>639258</v>
+        <v>373686</v>
       </c>
       <c r="C64" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D64" t="n">
         <v>0</v>
@@ -3371,14 +3333,14 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Shakeel Ahmed</t>
+          <t>Shehla Noor</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>373686</v>
+        <v>373650</v>
       </c>
       <c r="C65" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D65" t="n">
         <v>0</v>
@@ -3402,14 +3364,14 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Syed Haider Abbas</t>
+          <t>Sidra Khan</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>373713</v>
+        <v>373645</v>
       </c>
       <c r="C66" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D66" t="n">
         <v>0</v>
@@ -3433,31 +3395,62 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
+          <t>Syed Haider Abbas</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>373713</v>
+      </c>
+      <c r="C67" t="n">
+        <v>2</v>
+      </c>
+      <c r="D67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" t="n">
+        <v>0</v>
+      </c>
+      <c r="I67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
           <t>Usman Ali</t>
         </is>
       </c>
-      <c r="B67" t="n">
+      <c r="B68" t="n">
         <v>373687</v>
       </c>
-      <c r="C67" t="n">
+      <c r="C68" t="n">
         <v>8</v>
       </c>
-      <c r="D67" t="n">
-        <v>0</v>
-      </c>
-      <c r="E67" t="n">
-        <v>0</v>
-      </c>
-      <c r="F67" t="n">
-        <v>0</v>
-      </c>
-      <c r="G67" t="n">
-        <v>0</v>
-      </c>
-      <c r="H67" t="n">
-        <v>0</v>
-      </c>
-      <c r="I67" t="n">
+      <c r="D68" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update error log and tracking survey files for improved data accuracy
- Updated Daily_Error_Log.xlsx, Enumerator_Performance.xlsx, and Weekly_QA_Summary.xlsx to reflect the latest error metrics.
- Removed temporary file ~$Tracking_Survey_NewSample.xlsx to clean up the directory.
- Updated Tracking_Survey_NewSample.xlsx to ensure it contains the most recent data changes.
</commit_message>
<xml_diff>
--- a/Error_log/Enumerator_Performance.xlsx
+++ b/Error_log/Enumerator_Performance.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="performance" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="performance_pct" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="performance" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="performance_pct" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -35,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -43,12 +46,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -414,31 +426,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Enumerator Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Enumerator ID</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Total Issues</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Critical Issues</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Flag Issues</t>
         </is>
@@ -452,295 +464,295 @@
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
-        <v>2250</v>
+        <v>2437</v>
       </c>
       <c r="D2" t="n">
-        <v>2250</v>
+        <v>2435</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Shazia begum</t>
+          <t>Shafaq Zahra</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>373696</v>
+        <v>373646</v>
       </c>
       <c r="C3" t="n">
-        <v>126</v>
+        <v>149</v>
       </c>
       <c r="D3" t="n">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="E3" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Shazia begum</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>373646</v>
+        <v>373696</v>
       </c>
       <c r="C4" t="n">
-        <v>119</v>
+        <v>139</v>
       </c>
       <c r="D4" t="n">
-        <v>107</v>
+        <v>122</v>
       </c>
       <c r="E4" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>373642</v>
+        <v>373648</v>
       </c>
       <c r="C5" t="n">
-        <v>108</v>
+        <v>140</v>
       </c>
       <c r="D5" t="n">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="E5" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Asma Bibi</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>373648</v>
+        <v>373641</v>
       </c>
       <c r="C6" t="n">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="D6" t="n">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="E6" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Asma Bibi</t>
+          <t>Irum Ikram</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>373641</v>
+        <v>373642</v>
       </c>
       <c r="C7" t="n">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D7" t="n">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="E7" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Sadia Rustum</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>373649</v>
+        <v>373684</v>
       </c>
       <c r="C8" t="n">
-        <v>92</v>
+        <v>131</v>
       </c>
       <c r="D8" t="n">
-        <v>82</v>
+        <v>103</v>
       </c>
       <c r="E8" t="n">
-        <v>10</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Mehran Khan</t>
+          <t>Sadia Rustum</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>373684</v>
+        <v>373649</v>
       </c>
       <c r="C9" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="D9" t="n">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="E9" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Muhammad Yousaf</t>
+          <t>Zohra</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>373690</v>
+        <v>373692</v>
       </c>
       <c r="C10" t="n">
-        <v>70</v>
+        <v>178</v>
       </c>
       <c r="D10" t="n">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="E10" t="n">
-        <v>8</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Jaweria</t>
+          <t>Samara</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>163495</v>
+        <v>373658</v>
       </c>
       <c r="C11" t="n">
-        <v>56</v>
+        <v>178</v>
       </c>
       <c r="D11" t="n">
-        <v>55</v>
+        <v>80</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Naureen Khan</t>
+          <t>Rehana Bibi</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>373716</v>
+        <v>373691</v>
       </c>
       <c r="C12" t="n">
-        <v>53</v>
+        <v>174</v>
       </c>
       <c r="D12" t="n">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Javairia</t>
+          <t>Furqan Ullah Khan</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373651</v>
+        <v>373683</v>
       </c>
       <c r="C13" t="n">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="D13" t="n">
-        <v>51</v>
+        <v>65</v>
       </c>
       <c r="E13" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mahnoor</t>
+          <t>Khalida Bibi</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>373705</v>
+        <v>373673</v>
       </c>
       <c r="C14" t="n">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="D14" t="n">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="E14" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Furqan Ullah Khan</t>
+          <t>Muhammad Yousaf</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373683</v>
+        <v>373690</v>
       </c>
       <c r="C15" t="n">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="D15" t="n">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="E15" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Bushra Ayub</t>
+          <t>Javairia</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>373671</v>
+        <v>373651</v>
       </c>
       <c r="C16" t="n">
-        <v>49</v>
+        <v>73</v>
       </c>
       <c r="D16" t="n">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Khalida Bibi</t>
+          <t>Naureen Khan</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>373673</v>
+        <v>373716</v>
       </c>
       <c r="C17" t="n">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="D17" t="n">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
@@ -749,17 +761,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Asma Gull</t>
+          <t>Jaweria</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>373672</v>
+        <v>163495</v>
       </c>
       <c r="C18" t="n">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="D18" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="E18" t="n">
         <v>1</v>
@@ -768,55 +780,55 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Laiba Shams</t>
+          <t>Bushra Ayub</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>373706</v>
+        <v>373671</v>
       </c>
       <c r="C19" t="n">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="D19" t="n">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="E19" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Lati Khan</t>
+          <t>Mahnoor</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>373665</v>
+        <v>373705</v>
       </c>
       <c r="C20" t="n">
-        <v>35</v>
+        <v>53</v>
       </c>
       <c r="D20" t="n">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Naureen</t>
+          <t>Asma Gull</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>884887</v>
+        <v>373672</v>
       </c>
       <c r="C21" t="n">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="D21" t="n">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="E21" t="n">
         <v>4</v>
@@ -825,93 +837,93 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Lati Khan</t>
+          <t>Naureen khan</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>564273</v>
+        <v>453925</v>
       </c>
       <c r="C22" t="n">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="D22" t="n">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="E22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Summiya Hayat</t>
+          <t>Kainat</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>373710</v>
+        <v>373712</v>
       </c>
       <c r="C23" t="n">
-        <v>40</v>
+        <v>155</v>
       </c>
       <c r="D23" t="n">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="E23" t="n">
-        <v>13</v>
+        <v>96</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Naureen khan</t>
+          <t>Lati Khan</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>453925</v>
+        <v>564273</v>
       </c>
       <c r="C24" t="n">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="D24" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Muniba Shamim</t>
+          <t>Lati Khan</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>373659</v>
+        <v>373665</v>
       </c>
       <c r="C25" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="D25" t="n">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="E25" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Munawar Khan</t>
+          <t>Laiba Shams</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>373668</v>
+        <v>373706</v>
       </c>
       <c r="C26" t="n">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="D26" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="E26" t="n">
         <v>6</v>
@@ -920,131 +932,131 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Irum ikram</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>373692</v>
+        <v>541376</v>
       </c>
       <c r="C27" t="n">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="D27" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E27" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Lati khan</t>
+          <t>Naureen</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>671211</v>
+        <v>884887</v>
       </c>
       <c r="C28" t="n">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="D28" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E28" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Kainat</t>
+          <t>Summiya Hayat</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>373712</v>
+        <v>373710</v>
       </c>
       <c r="C29" t="n">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="D29" t="n">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="E29" t="n">
-        <v>36</v>
+        <v>13</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Samara</t>
+          <t>Muniba Shamim</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>373658</v>
+        <v>373659</v>
       </c>
       <c r="C30" t="n">
-        <v>62</v>
+        <v>32</v>
       </c>
       <c r="D30" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="E30" t="n">
-        <v>34</v>
+        <v>9</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Anum Gul</t>
+          <t>Munawar Khan</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>373656</v>
+        <v>373668</v>
       </c>
       <c r="C31" t="n">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="D31" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="E31" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Rehana Bibi</t>
+          <t>Lati khan</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>373691</v>
+        <v>671211</v>
       </c>
       <c r="C32" t="n">
-        <v>58</v>
+        <v>19</v>
       </c>
       <c r="D32" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="E32" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Alia Khan</t>
+          <t>Anum Gul</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>373681</v>
+        <v>373656</v>
       </c>
       <c r="C33" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="D33" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E33" t="n">
         <v>4</v>
@@ -1053,74 +1065,74 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Irum ikram</t>
+          <t>Alia Khan</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>541376</v>
+        <v>373681</v>
       </c>
       <c r="C34" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D34" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E34" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Ishaq Khan</t>
+          <t>Nillum Bibi</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>373699</v>
+        <v>373652</v>
       </c>
       <c r="C35" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D35" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E35" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Laiba Khan</t>
+          <t>Nazia</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>373653</v>
+        <v>373657</v>
       </c>
       <c r="C36" t="n">
         <v>8</v>
       </c>
       <c r="D36" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E36" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Nazia</t>
+          <t>Ishaq Khan</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>373657</v>
+        <v>373699</v>
       </c>
       <c r="C37" t="n">
+        <v>6</v>
+      </c>
+      <c r="D37" t="n">
         <v>5</v>
-      </c>
-      <c r="D37" t="n">
-        <v>4</v>
       </c>
       <c r="E37" t="n">
         <v>1</v>
@@ -1129,30 +1141,30 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Nillum Bibi</t>
+          <t>Laiba Khan</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>373652</v>
+        <v>373653</v>
       </c>
       <c r="C38" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D38" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E38" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Zain Ul Abideen</t>
+          <t>Shehla Noor</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>373667</v>
+        <v>373650</v>
       </c>
       <c r="C39" t="n">
         <v>3</v>
@@ -1167,17 +1179,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Muhammad Shahid Khan</t>
+          <t>Zain Ul Abideen</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>373662</v>
+        <v>373667</v>
       </c>
       <c r="C40" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D40" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E40" t="n">
         <v>0</v>
@@ -1186,68 +1198,68 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Chashm Gul</t>
+          <t>Muhammad Shahid Khan</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>373695</v>
+        <v>373662</v>
       </c>
       <c r="C41" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D41" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E41" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Muhammad naeem</t>
+          <t>Chashm Gul</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>571571</v>
+        <v>373695</v>
       </c>
       <c r="C42" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D42" t="n">
         <v>0</v>
       </c>
       <c r="E42" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Aisha Aman</t>
+          <t>Muhammad naeem</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>373704</v>
+        <v>571571</v>
       </c>
       <c r="C43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D43" t="n">
         <v>0</v>
       </c>
       <c r="E43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Mahnoorr</t>
+          <t>Aisha Aman</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>373670</v>
+        <v>373704</v>
       </c>
       <c r="C44" t="n">
         <v>1</v>
@@ -1262,11 +1274,11 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Muhammad Noor</t>
+          <t>Mahnoorr</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>373701</v>
+        <v>373670</v>
       </c>
       <c r="C45" t="n">
         <v>1</v>
@@ -1281,11 +1293,11 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Rahila Naaz</t>
+          <t>Muhammad Noor</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>373715</v>
+        <v>373701</v>
       </c>
       <c r="C46" t="n">
         <v>1</v>
@@ -1300,11 +1312,11 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Robina Shaheen</t>
+          <t>Rahila Naaz</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>373639</v>
+        <v>373715</v>
       </c>
       <c r="C47" t="n">
         <v>1</v>
@@ -1313,6 +1325,25 @@
         <v>0</v>
       </c>
       <c r="E47" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Robina Shaheen</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>373639</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1327,51 +1358,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I68"/>
+  <dimension ref="A1:I69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>enumerator_name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>enumerator_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>total_submissions</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>total_issues</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>critical_issues</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>flag_issues</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>error_pct</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>critical_error_pct</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>flag_error_pct</t>
         </is>
@@ -1390,19 +1421,19 @@
         <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="E2" t="n">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>1250</v>
+        <v>2200</v>
       </c>
       <c r="H2" t="n">
-        <v>1250</v>
+        <v>2200</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -1421,425 +1452,425 @@
         <v>9</v>
       </c>
       <c r="D3" t="n">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="E3" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G3" t="n">
-        <v>322.22</v>
+        <v>488.89</v>
       </c>
       <c r="H3" t="n">
-        <v>311.11</v>
+        <v>444.44</v>
       </c>
       <c r="I3" t="n">
-        <v>11.11</v>
+        <v>44.44</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lati khan</t>
+          <t>Irum ikram</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>671211</v>
+        <v>541376</v>
       </c>
       <c r="C4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D4" t="n">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="E4" t="n">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G4" t="n">
-        <v>211.11</v>
+        <v>450</v>
       </c>
       <c r="H4" t="n">
-        <v>211.11</v>
+        <v>387.5</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Irum ikram</t>
+          <t>Lati khan</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>541376</v>
+        <v>671211</v>
       </c>
       <c r="C5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D5" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E5" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="F5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>125</v>
+        <v>211.11</v>
       </c>
       <c r="H5" t="n">
-        <v>87.5</v>
+        <v>211.11</v>
       </c>
       <c r="I5" t="n">
-        <v>37.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Kainat</t>
+          <t>Zohra</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>373712</v>
+        <v>373692</v>
       </c>
       <c r="C6" t="n">
-        <v>69</v>
+        <v>101</v>
       </c>
       <c r="D6" t="n">
-        <v>61</v>
+        <v>178</v>
       </c>
       <c r="E6" t="n">
-        <v>14</v>
+        <v>85</v>
       </c>
       <c r="F6" t="n">
-        <v>36</v>
+        <v>85</v>
       </c>
       <c r="G6" t="n">
-        <v>88.41</v>
+        <v>176.24</v>
       </c>
       <c r="H6" t="n">
-        <v>20.29</v>
+        <v>84.16</v>
       </c>
       <c r="I6" t="n">
-        <v>52.17</v>
+        <v>84.16</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Naureen Khan</t>
+          <t>Rehana Bibi</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>373716</v>
+        <v>373691</v>
       </c>
       <c r="C7" t="n">
-        <v>62</v>
+        <v>111</v>
       </c>
       <c r="D7" t="n">
-        <v>53</v>
+        <v>174</v>
       </c>
       <c r="E7" t="n">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="G7" t="n">
-        <v>85.48</v>
+        <v>156.76</v>
       </c>
       <c r="H7" t="n">
-        <v>85.48</v>
+        <v>63.96</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>81.08</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Zohra</t>
+          <t>Kainat</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>373692</v>
+        <v>373712</v>
       </c>
       <c r="C8" t="n">
-        <v>65</v>
+        <v>104</v>
       </c>
       <c r="D8" t="n">
-        <v>55</v>
+        <v>155</v>
       </c>
       <c r="E8" t="n">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="F8" t="n">
-        <v>33</v>
+        <v>96</v>
       </c>
       <c r="G8" t="n">
-        <v>84.62</v>
+        <v>149.04</v>
       </c>
       <c r="H8" t="n">
-        <v>29.23</v>
+        <v>41.35</v>
       </c>
       <c r="I8" t="n">
-        <v>50.77</v>
+        <v>92.31</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Rehana Bibi</t>
+          <t>Samara</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>373691</v>
+        <v>373658</v>
       </c>
       <c r="C9" t="n">
-        <v>69</v>
+        <v>120</v>
       </c>
       <c r="D9" t="n">
-        <v>58</v>
+        <v>178</v>
       </c>
       <c r="E9" t="n">
-        <v>11</v>
+        <v>80</v>
       </c>
       <c r="F9" t="n">
-        <v>36</v>
+        <v>81</v>
       </c>
       <c r="G9" t="n">
-        <v>84.06</v>
+        <v>148.33</v>
       </c>
       <c r="H9" t="n">
-        <v>15.94</v>
+        <v>66.67</v>
       </c>
       <c r="I9" t="n">
-        <v>52.17</v>
+        <v>67.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Jaweria</t>
+          <t>Naureen Khan</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>163495</v>
+        <v>373716</v>
       </c>
       <c r="C10" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D10" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E10" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>82.34999999999999</v>
+        <v>82.86</v>
       </c>
       <c r="H10" t="n">
-        <v>80.88</v>
+        <v>82.86</v>
       </c>
       <c r="I10" t="n">
-        <v>1.47</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Shazia begum</t>
+          <t>Jaweria</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>373696</v>
+        <v>163495</v>
       </c>
       <c r="C11" t="n">
-        <v>160</v>
+        <v>68</v>
       </c>
       <c r="D11" t="n">
-        <v>126</v>
+        <v>56</v>
       </c>
       <c r="E11" t="n">
-        <v>112</v>
+        <v>55</v>
       </c>
       <c r="F11" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>78.75</v>
+        <v>82.34999999999999</v>
       </c>
       <c r="H11" t="n">
-        <v>70</v>
+        <v>80.88</v>
       </c>
       <c r="I11" t="n">
-        <v>8.75</v>
+        <v>1.47</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Shafaq Zahra</t>
+          <t>Shazia begum</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>373646</v>
+        <v>373696</v>
       </c>
       <c r="C12" t="n">
-        <v>153</v>
+        <v>179</v>
       </c>
       <c r="D12" t="n">
-        <v>119</v>
+        <v>139</v>
       </c>
       <c r="E12" t="n">
-        <v>107</v>
+        <v>122</v>
       </c>
       <c r="F12" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G12" t="n">
-        <v>77.78</v>
+        <v>77.65000000000001</v>
       </c>
       <c r="H12" t="n">
-        <v>69.93000000000001</v>
+        <v>68.16</v>
       </c>
       <c r="I12" t="n">
-        <v>7.84</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Asma Bibi</t>
+          <t>Shazia Bibi</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>373641</v>
+        <v>373648</v>
       </c>
       <c r="C13" t="n">
-        <v>150</v>
+        <v>189</v>
       </c>
       <c r="D13" t="n">
-        <v>113</v>
+        <v>140</v>
       </c>
       <c r="E13" t="n">
-        <v>99</v>
+        <v>117</v>
       </c>
       <c r="F13" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="G13" t="n">
-        <v>75.33</v>
+        <v>74.06999999999999</v>
       </c>
       <c r="H13" t="n">
-        <v>66</v>
+        <v>61.9</v>
       </c>
       <c r="I13" t="n">
-        <v>9.33</v>
+        <v>12.17</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Samara</t>
+          <t>Irum Ikram</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>373658</v>
+        <v>373642</v>
       </c>
       <c r="C14" t="n">
-        <v>83</v>
+        <v>150</v>
       </c>
       <c r="D14" t="n">
-        <v>62</v>
+        <v>109</v>
       </c>
       <c r="E14" t="n">
-        <v>13</v>
+        <v>105</v>
       </c>
       <c r="F14" t="n">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="G14" t="n">
-        <v>74.7</v>
+        <v>72.67</v>
       </c>
       <c r="H14" t="n">
-        <v>15.66</v>
+        <v>70</v>
       </c>
       <c r="I14" t="n">
-        <v>40.96</v>
+        <v>2.67</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Shazia Bibi</t>
+          <t>Shafaq Zahra</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>373648</v>
+        <v>373646</v>
       </c>
       <c r="C15" t="n">
-        <v>164</v>
+        <v>207</v>
       </c>
       <c r="D15" t="n">
-        <v>120</v>
+        <v>149</v>
       </c>
       <c r="E15" t="n">
-        <v>101</v>
+        <v>133</v>
       </c>
       <c r="F15" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G15" t="n">
-        <v>73.17</v>
+        <v>71.98</v>
       </c>
       <c r="H15" t="n">
-        <v>61.59</v>
+        <v>64.25</v>
       </c>
       <c r="I15" t="n">
-        <v>11.59</v>
+        <v>7.73</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Irum Ikram</t>
+          <t>Asma Bibi</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>373642</v>
+        <v>373641</v>
       </c>
       <c r="C16" t="n">
-        <v>149</v>
+        <v>187</v>
       </c>
       <c r="D16" t="n">
-        <v>108</v>
+        <v>134</v>
       </c>
       <c r="E16" t="n">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="F16" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="G16" t="n">
-        <v>72.48</v>
+        <v>71.66</v>
       </c>
       <c r="H16" t="n">
-        <v>69.8</v>
+        <v>59.89</v>
       </c>
       <c r="I16" t="n">
-        <v>2.68</v>
+        <v>11.76</v>
       </c>
     </row>
     <row r="17">
@@ -1852,118 +1883,118 @@
         <v>373649</v>
       </c>
       <c r="C17" t="n">
-        <v>130</v>
+        <v>152</v>
       </c>
       <c r="D17" t="n">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="E17" t="n">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="F17" t="n">
         <v>10</v>
       </c>
       <c r="G17" t="n">
-        <v>70.77</v>
+        <v>69.73999999999999</v>
       </c>
       <c r="H17" t="n">
-        <v>63.08</v>
+        <v>63.16</v>
       </c>
       <c r="I17" t="n">
-        <v>7.69</v>
+        <v>6.58</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Lati Khan</t>
+          <t>Mehran Khan</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>373665</v>
+        <v>373684</v>
       </c>
       <c r="C18" t="n">
-        <v>52</v>
+        <v>196</v>
       </c>
       <c r="D18" t="n">
-        <v>35</v>
+        <v>131</v>
       </c>
       <c r="E18" t="n">
-        <v>34</v>
+        <v>103</v>
       </c>
       <c r="F18" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="G18" t="n">
-        <v>67.31</v>
+        <v>66.84</v>
       </c>
       <c r="H18" t="n">
-        <v>65.38</v>
+        <v>52.55</v>
       </c>
       <c r="I18" t="n">
-        <v>1.92</v>
+        <v>14.29</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Javairia</t>
+          <t>Lati Khan</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>373651</v>
+        <v>373665</v>
       </c>
       <c r="C19" t="n">
-        <v>95</v>
+        <v>60</v>
       </c>
       <c r="D19" t="n">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="E19" t="n">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="F19" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="G19" t="n">
-        <v>65.26000000000001</v>
+        <v>66.67</v>
       </c>
       <c r="H19" t="n">
-        <v>53.68</v>
+        <v>61.67</v>
       </c>
       <c r="I19" t="n">
-        <v>11.58</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Mehran Khan</t>
+          <t>Javairia</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>373684</v>
+        <v>373651</v>
       </c>
       <c r="C20" t="n">
-        <v>158</v>
+        <v>120</v>
       </c>
       <c r="D20" t="n">
-        <v>102</v>
+        <v>73</v>
       </c>
       <c r="E20" t="n">
-        <v>79</v>
+        <v>60</v>
       </c>
       <c r="F20" t="n">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="G20" t="n">
-        <v>64.56</v>
+        <v>60.83</v>
       </c>
       <c r="H20" t="n">
         <v>50</v>
       </c>
       <c r="I20" t="n">
-        <v>14.56</v>
+        <v>10.83</v>
       </c>
     </row>
     <row r="21">
@@ -2193,25 +2224,25 @@
         <v>373671</v>
       </c>
       <c r="C28" t="n">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="D28" t="n">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="E28" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="F28" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G28" t="n">
-        <v>39.52</v>
+        <v>39.86</v>
       </c>
       <c r="H28" t="n">
-        <v>37.9</v>
+        <v>36.96</v>
       </c>
       <c r="I28" t="n">
-        <v>1.61</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="29">
@@ -2224,87 +2255,87 @@
         <v>373683</v>
       </c>
       <c r="C29" t="n">
-        <v>142</v>
+        <v>184</v>
       </c>
       <c r="D29" t="n">
-        <v>52</v>
+        <v>73</v>
       </c>
       <c r="E29" t="n">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="F29" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G29" t="n">
-        <v>36.62</v>
+        <v>39.67</v>
       </c>
       <c r="H29" t="n">
-        <v>33.8</v>
+        <v>35.33</v>
       </c>
       <c r="I29" t="n">
-        <v>2.82</v>
+        <v>4.35</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Asma Gull</t>
+          <t>Khalida Bibi</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>373672</v>
+        <v>373673</v>
       </c>
       <c r="C30" t="n">
-        <v>129</v>
+        <v>177</v>
       </c>
       <c r="D30" t="n">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="E30" t="n">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="F30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>35.66</v>
+        <v>35.59</v>
       </c>
       <c r="H30" t="n">
-        <v>34.88</v>
+        <v>35.59</v>
       </c>
       <c r="I30" t="n">
-        <v>0.78</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Khalida Bibi</t>
+          <t>Asma Gull</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>373673</v>
+        <v>373672</v>
       </c>
       <c r="C31" t="n">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="D31" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E31" t="n">
         <v>47</v>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G31" t="n">
-        <v>33.57</v>
+        <v>35.42</v>
       </c>
       <c r="H31" t="n">
-        <v>33.57</v>
+        <v>32.64</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>2.78</v>
       </c>
     </row>
     <row r="32">
@@ -2434,73 +2465,73 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Anum Gul</t>
+          <t>Shehla Noor</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>373656</v>
+        <v>373650</v>
       </c>
       <c r="C36" t="n">
-        <v>97</v>
+        <v>14</v>
       </c>
       <c r="D36" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="E36" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="F36" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>17.53</v>
+        <v>21.43</v>
       </c>
       <c r="H36" t="n">
-        <v>13.4</v>
+        <v>21.43</v>
       </c>
       <c r="I36" t="n">
-        <v>4.12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Muhammad Noor</t>
+          <t>Anum Gul</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>373701</v>
+        <v>373656</v>
       </c>
       <c r="C37" t="n">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="E37" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="F37" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G37" t="n">
-        <v>12.5</v>
+        <v>17.48</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>13.59</v>
       </c>
       <c r="I37" t="n">
-        <v>12.5</v>
+        <v>3.88</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Robina Shaheen</t>
+          <t>Muhammad Noor</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>373639</v>
+        <v>373701</v>
       </c>
       <c r="C38" t="n">
         <v>8</v>
@@ -2527,94 +2558,94 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Alia Khan</t>
+          <t>Robina Shaheen</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>373681</v>
+        <v>373639</v>
       </c>
       <c r="C39" t="n">
-        <v>113</v>
+        <v>8</v>
       </c>
       <c r="D39" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G39" t="n">
-        <v>11.5</v>
+        <v>12.5</v>
       </c>
       <c r="H39" t="n">
-        <v>7.96</v>
+        <v>0</v>
       </c>
       <c r="I39" t="n">
-        <v>3.54</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Aisha Aman</t>
+          <t>Alia Khan</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>373704</v>
+        <v>373681</v>
       </c>
       <c r="C40" t="n">
-        <v>11</v>
+        <v>129</v>
       </c>
       <c r="D40" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E40" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F40" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G40" t="n">
-        <v>9.09</v>
+        <v>10.08</v>
       </c>
       <c r="H40" t="n">
-        <v>0</v>
+        <v>6.98</v>
       </c>
       <c r="I40" t="n">
-        <v>9.09</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Laiba Khan</t>
+          <t>Aisha Aman</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>373653</v>
+        <v>373704</v>
       </c>
       <c r="C41" t="n">
-        <v>104</v>
+        <v>11</v>
       </c>
       <c r="D41" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G41" t="n">
-        <v>7.69</v>
+        <v>9.09</v>
       </c>
       <c r="H41" t="n">
-        <v>3.85</v>
+        <v>0</v>
       </c>
       <c r="I41" t="n">
-        <v>3.85</v>
+        <v>9.09</v>
       </c>
     </row>
     <row r="42">
@@ -2651,32 +2682,32 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Nazia</t>
+          <t>Laiba Khan</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>373657</v>
+        <v>373653</v>
       </c>
       <c r="C43" t="n">
-        <v>97</v>
+        <v>121</v>
       </c>
       <c r="D43" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E43" t="n">
         <v>4</v>
       </c>
       <c r="F43" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G43" t="n">
-        <v>5.15</v>
+        <v>6.61</v>
       </c>
       <c r="H43" t="n">
-        <v>4.12</v>
+        <v>3.31</v>
       </c>
       <c r="I43" t="n">
-        <v>1.03</v>
+        <v>3.31</v>
       </c>
     </row>
     <row r="44">
@@ -2689,100 +2720,100 @@
         <v>373652</v>
       </c>
       <c r="C44" t="n">
-        <v>119</v>
+        <v>169</v>
       </c>
       <c r="D44" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E44" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F44" t="n">
         <v>3</v>
       </c>
       <c r="G44" t="n">
-        <v>5.04</v>
+        <v>5.92</v>
       </c>
       <c r="H44" t="n">
-        <v>2.52</v>
+        <v>4.14</v>
       </c>
       <c r="I44" t="n">
-        <v>2.52</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Ishaq Khan</t>
+          <t>Nazia</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>373699</v>
+        <v>373657</v>
       </c>
       <c r="C45" t="n">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="D45" t="n">
+        <v>8</v>
+      </c>
+      <c r="E45" t="n">
         <v>6</v>
       </c>
-      <c r="E45" t="n">
-        <v>5</v>
-      </c>
       <c r="F45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G45" t="n">
-        <v>4.51</v>
+        <v>5.56</v>
       </c>
       <c r="H45" t="n">
-        <v>3.76</v>
+        <v>4.17</v>
       </c>
       <c r="I45" t="n">
-        <v>0.75</v>
+        <v>1.39</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Gul Rukh</t>
+          <t>Ishaq Khan</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>373644</v>
+        <v>373699</v>
       </c>
       <c r="C46" t="n">
+        <v>170</v>
+      </c>
+      <c r="D46" t="n">
         <v>6</v>
       </c>
-      <c r="D46" t="n">
-        <v>0</v>
-      </c>
       <c r="E46" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G46" t="n">
-        <v>0</v>
+        <v>3.53</v>
       </c>
       <c r="H46" t="n">
-        <v>0</v>
+        <v>2.94</v>
       </c>
       <c r="I46" t="n">
-        <v>0</v>
+        <v>0.59</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Hijab Zahra</t>
+          <t>Gul Rukh</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>373637</v>
+        <v>373644</v>
       </c>
       <c r="C47" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D47" t="n">
         <v>0</v>
@@ -2806,14 +2837,14 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Iqra Bibi</t>
+          <t>Hijab Zahra</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>373708</v>
+        <v>373637</v>
       </c>
       <c r="C48" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D48" t="n">
         <v>0</v>
@@ -2837,14 +2868,14 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Irum ikram (duplicate name received from listed_girl_tracking_survey on June 29, 2026 12:08 UTC+00:00; submission key: uuid:b700a976-75ee-467c-87e9-1d5163ec238d)</t>
+          <t>Iqra Bibi</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>541376</v>
+        <v>373708</v>
       </c>
       <c r="C49" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="D49" t="n">
         <v>0</v>
@@ -2868,14 +2899,14 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Lati Khan (duplicate name received from listed_girl_tracking_survey on June 28, 2026 10:43 UTC+00:00; submission key: uuid:e4e89d53-e5be-40ff-bb2c-fa94c0d50011)</t>
+          <t>Irum ikram (duplicate name received from listed_girl_tracking_survey on June 29, 2026 12:08 UTC+00:00; submission key: uuid:b700a976-75ee-467c-87e9-1d5163ec238d)</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>564273</v>
+        <v>541376</v>
       </c>
       <c r="C50" t="n">
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="D50" t="n">
         <v>0</v>
@@ -2899,14 +2930,14 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Lati khan</t>
+          <t>Lati Khan (duplicate name received from listed_girl_tracking_survey on June 28, 2026 10:43 UTC+00:00; submission key: uuid:e4e89d53-e5be-40ff-bb2c-fa94c0d50011)</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>652938</v>
+        <v>564273</v>
       </c>
       <c r="C51" t="n">
-        <v>11</v>
+        <v>55</v>
       </c>
       <c r="D51" t="n">
         <v>0</v>
@@ -2930,14 +2961,14 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Lati khan (duplicate name received from listed_girl_tracking_survey_new_sample on July 4, 2026 14:31 UTC+00:00; submission key: uuid:6316d214-c458-4786-937a-bd81b08c15c5)</t>
+          <t>Lati khan</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>671211</v>
+        <v>652938</v>
       </c>
       <c r="C52" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D52" t="n">
         <v>0</v>
@@ -2961,14 +2992,14 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Muhammad Naeem</t>
+          <t>Lati khan (duplicate name received from listed_girl_tracking_survey_new_sample on July 4, 2026 14:31 UTC+00:00; submission key: uuid:6316d214-c458-4786-937a-bd81b08c15c5)</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>373694</v>
+        <v>671211</v>
       </c>
       <c r="C53" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="D53" t="n">
         <v>0</v>
@@ -2992,14 +3023,14 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Muhammad Usman</t>
+          <t>Muhammad Naeem</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>373666</v>
+        <v>373694</v>
       </c>
       <c r="C54" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="D54" t="n">
         <v>0</v>
@@ -3023,14 +3054,14 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Muhammad Waseem</t>
+          <t>Muhammad Usman</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>373689</v>
+        <v>373666</v>
       </c>
       <c r="C55" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="D55" t="n">
         <v>0</v>
@@ -3054,14 +3085,14 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Muhammad naeem (duplicate name received from primary_school_listing_survey on February 14, 2026 14:38 UTC+00:00; submission key: uuid:5f0e427e-5fd2-4474-be64-ae5f2c4617a2)</t>
+          <t>Muhammad Waseem</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>571571</v>
+        <v>373689</v>
       </c>
       <c r="C56" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="D56" t="n">
         <v>0</v>
@@ -3085,14 +3116,14 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Nadia bibi</t>
+          <t>Muhammad naeem (duplicate name received from primary_school_listing_survey on February 14, 2026 14:38 UTC+00:00; submission key: uuid:5f0e427e-5fd2-4474-be64-ae5f2c4617a2)</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>373669</v>
+        <v>571571</v>
       </c>
       <c r="C57" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D57" t="n">
         <v>0</v>
@@ -3116,14 +3147,14 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Naureen khan (duplicate name received from listed_girl_tracking_survey_new_sample on July 7, 2026 14:41 UTC+00:00; submission key: uuid:bbf56e1f-36f5-4ebf-9e0f-df83015a0871)</t>
+          <t>Nadia bibi</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>453925</v>
+        <v>373669</v>
       </c>
       <c r="C58" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="D58" t="n">
         <v>0</v>
@@ -3147,14 +3178,14 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Saba Ramzan</t>
+          <t>Naureen khan (duplicate name received from listed_girl_tracking_survey_new_sample on July 7, 2026 14:41 UTC+00:00; submission key: uuid:bbf56e1f-36f5-4ebf-9e0f-df83015a0871)</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>373703</v>
+        <v>453925</v>
       </c>
       <c r="C59" t="n">
-        <v>13</v>
+        <v>53</v>
       </c>
       <c r="D59" t="n">
         <v>0</v>
@@ -3178,14 +3209,14 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Sadia rustum</t>
+          <t>Saba Ramzan</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>852541</v>
+        <v>373703</v>
       </c>
       <c r="C60" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="D60" t="n">
         <v>0</v>
@@ -3209,14 +3240,14 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Sajjad Khan</t>
+          <t>Sadia rustum</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>373700</v>
+        <v>852541</v>
       </c>
       <c r="C61" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D61" t="n">
         <v>0</v>
@@ -3240,14 +3271,14 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Samreen</t>
+          <t>Sajjad Khan</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>373711</v>
+        <v>373700</v>
       </c>
       <c r="C62" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D62" t="n">
         <v>0</v>
@@ -3275,10 +3306,10 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>639258</v>
+        <v>373711</v>
       </c>
       <c r="C63" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D63" t="n">
         <v>0</v>
@@ -3302,14 +3333,14 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Shakeel Ahmed</t>
+          <t>Samreen</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>373686</v>
+        <v>639258</v>
       </c>
       <c r="C64" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D64" t="n">
         <v>0</v>
@@ -3333,14 +3364,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Shehla Noor</t>
-        </is>
-      </c>
-      <c r="B65" t="n">
-        <v>373650</v>
-      </c>
+          <t>Shafaq.zahra</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr"/>
       <c r="C65" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D65" t="n">
         <v>0</v>
@@ -3364,14 +3393,14 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Sidra Khan</t>
+          <t>Shakeel Ahmed</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>373645</v>
+        <v>373686</v>
       </c>
       <c r="C66" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D66" t="n">
         <v>0</v>
@@ -3395,14 +3424,14 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Syed Haider Abbas</t>
+          <t>Sidra Khan</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>373713</v>
+        <v>373645</v>
       </c>
       <c r="C67" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D67" t="n">
         <v>0</v>
@@ -3426,31 +3455,62 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
+          <t>Syed Haider Abbas</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>373713</v>
+      </c>
+      <c r="C68" t="n">
+        <v>2</v>
+      </c>
+      <c r="D68" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
           <t>Usman Ali</t>
         </is>
       </c>
-      <c r="B68" t="n">
+      <c r="B69" t="n">
         <v>373687</v>
       </c>
-      <c r="C68" t="n">
+      <c r="C69" t="n">
         <v>8</v>
       </c>
-      <c r="D68" t="n">
-        <v>0</v>
-      </c>
-      <c r="E68" t="n">
-        <v>0</v>
-      </c>
-      <c r="F68" t="n">
-        <v>0</v>
-      </c>
-      <c r="G68" t="n">
-        <v>0</v>
-      </c>
-      <c r="H68" t="n">
-        <v>0</v>
-      </c>
-      <c r="I68" t="n">
+      <c r="D69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" t="n">
+        <v>0</v>
+      </c>
+      <c r="I69" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>